<commit_message>
fix bug update department
</commit_message>
<xml_diff>
--- a/docs/members/linhdn/Professional_Bug_Tracker_Template.xlsx
+++ b/docs/members/linhdn/Professional_Bug_Tracker_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dowload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KÌ 5\SWP\hireflow-api\RetireManagement\SWP_RMS_Group-2\docs\members\linhdn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72C1335-D8F0-4F5B-AAB1-0A6209F55F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBFDBA3-7340-468B-A972-48500F2FEC75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="204">
   <si>
     <t>BUG QUALITY DASHBOARD</t>
   </si>
@@ -644,6 +644,12 @@
   </si>
   <si>
     <t>Lỗi FE khi bấm đóng dợt tuyể</t>
+  </si>
+  <si>
+    <t>B07</t>
+  </si>
+  <si>
+    <t>lỗi  mất kết nối sever</t>
   </si>
 </sst>
 </file>
@@ -944,14 +950,59 @@
     <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -977,61 +1028,13 @@
     <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1041,13 +1044,16 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1344,7 +1350,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2</c:v>
@@ -1520,7 +1526,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2</c:v>
@@ -1967,66 +1973,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
     </row>
     <row r="2" spans="1:12" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
     </row>
     <row r="3" spans="1:12" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
     </row>
     <row r="4" spans="1:12" ht="28" customHeight="1">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
     </row>
     <row r="5" spans="1:12" ht="14.5">
       <c r="A5" s="11"/>
@@ -2043,80 +2049,80 @@
       <c r="L5" s="11"/>
     </row>
     <row r="6" spans="1:12" ht="29" customHeight="1">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="26" t="s">
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="28" t="s">
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="30" t="s">
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="30"/>
-      <c r="L6" s="30"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="45"/>
     </row>
     <row r="7" spans="1:12" ht="24" customHeight="1">
-      <c r="A7" s="25">
+      <c r="A7" s="40">
         <f>COUNTIF('Bug Log'!$A$7:$A$306,"&lt;&gt;")</f>
-        <v>7</v>
-      </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="27">
+        <v>8</v>
+      </c>
+      <c r="B7" s="40"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="42">
         <f>COUNTIF('Bug Log'!$A$7:$A$306,"&lt;&gt;")-COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Closed")-COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Duplicate")-COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Won't Fix")</f>
-        <v>7</v>
-      </c>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="29">
+        <v>8</v>
+      </c>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="44">
         <f ca="1">COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$Q$7:$Q$306,"Quá hạn")</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="31">
+        <v>2</v>
+      </c>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="46">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Closed")</f>
         <v>0</v>
       </c>
-      <c r="K7" s="31"/>
-      <c r="L7" s="31"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
     </row>
     <row r="8" spans="1:12" ht="24" customHeight="1">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="31"/>
+      <c r="A8" s="40"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="46"/>
+      <c r="K8" s="46"/>
+      <c r="L8" s="46"/>
     </row>
     <row r="9" spans="1:12" ht="24" customHeight="1">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
+      <c r="A9" s="40"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="46"/>
+      <c r="K9" s="46"/>
+      <c r="L9" s="46"/>
     </row>
     <row r="10" spans="1:12" ht="14.5">
       <c r="A10" s="11"/>
@@ -2148,16 +2154,16 @@
       </c>
       <c r="H11" s="36"/>
       <c r="I11" s="36"/>
-      <c r="J11" s="39" t="s">
+      <c r="J11" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="K11" s="39"/>
-      <c r="L11" s="39"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
     </row>
     <row r="12" spans="1:12" ht="24" customHeight="1">
       <c r="A12" s="33">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$E$7:$E$306,"Blocker")+COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$E$7:$E$306,"Critical")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="33"/>
@@ -2173,12 +2179,12 @@
       </c>
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
-      <c r="J12" s="40">
+      <c r="J12" s="30">
         <f ca="1">IFERROR(AVERAGE('Bug Log'!$P$7:$P$306),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
+        <v>7</v>
+      </c>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
     </row>
     <row r="13" spans="1:12" ht="24" customHeight="1">
       <c r="A13" s="33"/>
@@ -2190,9 +2196,9 @@
       <c r="G13" s="38"/>
       <c r="H13" s="38"/>
       <c r="I13" s="38"/>
-      <c r="J13" s="41"/>
-      <c r="K13" s="41"/>
-      <c r="L13" s="41"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
     </row>
     <row r="14" spans="1:12" ht="24" customHeight="1">
       <c r="A14" s="33"/>
@@ -2204,9 +2210,9 @@
       <c r="G14" s="38"/>
       <c r="H14" s="38"/>
       <c r="I14" s="38"/>
-      <c r="J14" s="41"/>
-      <c r="K14" s="41"/>
-      <c r="L14" s="41"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
     </row>
     <row r="15" spans="1:12" ht="14.5">
       <c r="A15" s="11"/>
@@ -2223,24 +2229,24 @@
       <c r="L15" s="11"/>
     </row>
     <row r="16" spans="1:12" ht="31" customHeight="1">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
       <c r="E16" s="11"/>
-      <c r="F16" s="42" t="s">
+      <c r="F16" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42" t="s">
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="K16" s="42"/>
-      <c r="L16" s="42"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="28"/>
     </row>
     <row r="17" spans="1:12" ht="25" customHeight="1">
       <c r="A17" s="12" t="s">
@@ -2280,11 +2286,11 @@
       </c>
       <c r="B18" s="14">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,A18)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" s="15">
         <f t="shared" ref="C18:C26" si="0">IFERROR(B18/$A$7,0)</f>
-        <v>0.7142857142857143</v>
+        <v>0.75</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
@@ -2293,11 +2299,11 @@
       </c>
       <c r="G18" s="11">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$E$7:$E$306,F18)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="13">
         <f>IFERROR(G18/$A$7,0)</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I18" s="11"/>
       <c r="J18" s="11" t="s">
@@ -2305,11 +2311,11 @@
       </c>
       <c r="K18" s="11">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$F$7:$F$306,J18)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" s="13">
         <f>IFERROR(K18/$A$7,0)</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="25" customHeight="1">
@@ -2322,7 +2328,7 @@
       </c>
       <c r="C19" s="15">
         <f t="shared" si="0"/>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
@@ -2335,7 +2341,7 @@
       </c>
       <c r="H19" s="13">
         <f>IFERROR(G19/$A$7,0)</f>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
       <c r="I19" s="11"/>
       <c r="J19" s="11" t="s">
@@ -2347,7 +2353,7 @@
       </c>
       <c r="L19" s="13">
         <f>IFERROR(K19/$A$7,0)</f>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="25" customHeight="1">
@@ -2373,7 +2379,7 @@
       </c>
       <c r="H20" s="13">
         <f>IFERROR(G20/$A$7,0)</f>
-        <v>0.14285714285714285</v>
+        <v>0.125</v>
       </c>
       <c r="I20" s="11"/>
       <c r="J20" s="11" t="s">
@@ -2385,7 +2391,7 @@
       </c>
       <c r="L20" s="13">
         <f>IFERROR(K20/$A$7,0)</f>
-        <v>0.42857142857142855</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="25" customHeight="1">
@@ -2411,7 +2417,7 @@
       </c>
       <c r="H21" s="13">
         <f>IFERROR(G21/$A$7,0)</f>
-        <v>0.5714285714285714</v>
+        <v>0.5</v>
       </c>
       <c r="I21" s="11"/>
       <c r="J21" s="11" t="s">
@@ -2423,7 +2429,7 @@
       </c>
       <c r="L21" s="13">
         <f>IFERROR(K21/$A$7,0)</f>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="25" customHeight="1">
@@ -2559,22 +2565,22 @@
       <c r="L27" s="11"/>
     </row>
     <row r="28" spans="1:12" ht="31" customHeight="1">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42" t="s">
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="H28" s="42"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="42"/>
-      <c r="K28" s="42"/>
-      <c r="L28" s="42"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="28"/>
     </row>
     <row r="29" spans="1:12" ht="14.5">
       <c r="A29" s="11"/>
@@ -2829,22 +2835,22 @@
       <c r="L46" s="11"/>
     </row>
     <row r="47" spans="1:12" ht="31" customHeight="1">
-      <c r="A47" s="42" t="s">
+      <c r="A47" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="B47" s="42"/>
-      <c r="C47" s="42"/>
-      <c r="D47" s="42"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
       <c r="E47" s="11"/>
-      <c r="F47" s="42" t="s">
+      <c r="F47" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="G47" s="42"/>
-      <c r="H47" s="42"/>
-      <c r="I47" s="42"/>
-      <c r="J47" s="42"/>
-      <c r="K47" s="42"/>
-      <c r="L47" s="42"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="28"/>
+      <c r="I47" s="28"/>
+      <c r="J47" s="28"/>
+      <c r="K47" s="28"/>
+      <c r="L47" s="28"/>
     </row>
     <row r="48" spans="1:12" ht="27" customHeight="1">
       <c r="A48" s="12" t="s">
@@ -2880,15 +2886,15 @@
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="11"/>
-      <c r="F49" s="23" t="s">
+      <c r="F49" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="G49" s="23"/>
-      <c r="H49" s="23"/>
-      <c r="I49" s="23"/>
-      <c r="J49" s="23"/>
-      <c r="K49" s="23"/>
-      <c r="L49" s="23"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="26"/>
+      <c r="I49" s="26"/>
+      <c r="J49" s="26"/>
+      <c r="K49" s="26"/>
+      <c r="L49" s="26"/>
     </row>
     <row r="50" spans="1:12" ht="20" customHeight="1">
       <c r="A50" s="11" t="s">
@@ -2904,13 +2910,13 @@
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="11"/>
-      <c r="F50" s="23"/>
-      <c r="G50" s="23"/>
-      <c r="H50" s="23"/>
-      <c r="I50" s="23"/>
-      <c r="J50" s="23"/>
-      <c r="K50" s="23"/>
-      <c r="L50" s="23"/>
+      <c r="F50" s="26"/>
+      <c r="G50" s="26"/>
+      <c r="H50" s="26"/>
+      <c r="I50" s="26"/>
+      <c r="J50" s="26"/>
+      <c r="K50" s="26"/>
+      <c r="L50" s="26"/>
     </row>
     <row r="51" spans="1:12" ht="24" customHeight="1">
       <c r="A51" s="11" t="s">
@@ -2922,7 +2928,7 @@
       </c>
       <c r="C51" s="13">
         <f t="shared" si="1"/>
-        <v>0.14285714285714285</v>
+        <v>0.125</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="11"/>
@@ -2948,15 +2954,15 @@
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="11"/>
-      <c r="F52" s="43" t="s">
+      <c r="F52" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="G52" s="43"/>
-      <c r="H52" s="43"/>
-      <c r="I52" s="43"/>
-      <c r="J52" s="43"/>
-      <c r="K52" s="43"/>
-      <c r="L52" s="43"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="25"/>
+      <c r="I52" s="25"/>
+      <c r="J52" s="25"/>
+      <c r="K52" s="25"/>
+      <c r="L52" s="25"/>
     </row>
     <row r="53" spans="1:12" ht="20" customHeight="1">
       <c r="A53" s="11" t="s">
@@ -2972,13 +2978,13 @@
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="11"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="43"/>
-      <c r="I53" s="43"/>
-      <c r="J53" s="43"/>
-      <c r="K53" s="43"/>
-      <c r="L53" s="43"/>
+      <c r="F53" s="25"/>
+      <c r="G53" s="25"/>
+      <c r="H53" s="25"/>
+      <c r="I53" s="25"/>
+      <c r="J53" s="25"/>
+      <c r="K53" s="25"/>
+      <c r="L53" s="25"/>
     </row>
     <row r="54" spans="1:12" ht="24" customHeight="1">
       <c r="A54" s="11" t="s">
@@ -2990,7 +2996,7 @@
       </c>
       <c r="C54" s="13">
         <f t="shared" si="1"/>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="11"/>
@@ -3012,19 +3018,19 @@
       </c>
       <c r="C55" s="13">
         <f t="shared" si="1"/>
-        <v>0.42857142857142855</v>
+        <v>0.375</v>
       </c>
       <c r="D55" s="11"/>
       <c r="E55" s="11"/>
-      <c r="F55" s="23" t="s">
+      <c r="F55" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="G55" s="23"/>
-      <c r="H55" s="23"/>
-      <c r="I55" s="23"/>
-      <c r="J55" s="23"/>
-      <c r="K55" s="23"/>
-      <c r="L55" s="23"/>
+      <c r="G55" s="26"/>
+      <c r="H55" s="26"/>
+      <c r="I55" s="26"/>
+      <c r="J55" s="26"/>
+      <c r="K55" s="26"/>
+      <c r="L55" s="26"/>
     </row>
     <row r="56" spans="1:12" ht="20" customHeight="1">
       <c r="A56" s="11" t="s">
@@ -3040,13 +3046,13 @@
       </c>
       <c r="D56" s="11"/>
       <c r="E56" s="11"/>
-      <c r="F56" s="23"/>
-      <c r="G56" s="23"/>
-      <c r="H56" s="23"/>
-      <c r="I56" s="23"/>
-      <c r="J56" s="23"/>
-      <c r="K56" s="23"/>
-      <c r="L56" s="23"/>
+      <c r="F56" s="26"/>
+      <c r="G56" s="26"/>
+      <c r="H56" s="26"/>
+      <c r="I56" s="26"/>
+      <c r="J56" s="26"/>
+      <c r="K56" s="26"/>
+      <c r="L56" s="26"/>
     </row>
     <row r="57" spans="1:12" ht="24" customHeight="1">
       <c r="A57" s="11" t="s">
@@ -3058,7 +3064,7 @@
       </c>
       <c r="C57" s="13">
         <f t="shared" si="1"/>
-        <v>0.14285714285714285</v>
+        <v>0.125</v>
       </c>
       <c r="D57" s="11"/>
       <c r="E57" s="11"/>
@@ -3084,15 +3090,15 @@
       </c>
       <c r="D58" s="11"/>
       <c r="E58" s="11"/>
-      <c r="F58" s="43" t="s">
+      <c r="F58" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="G58" s="43"/>
-      <c r="H58" s="43"/>
-      <c r="I58" s="43"/>
-      <c r="J58" s="43"/>
-      <c r="K58" s="43"/>
-      <c r="L58" s="43"/>
+      <c r="G58" s="25"/>
+      <c r="H58" s="25"/>
+      <c r="I58" s="25"/>
+      <c r="J58" s="25"/>
+      <c r="K58" s="25"/>
+      <c r="L58" s="25"/>
     </row>
     <row r="59" spans="1:12" ht="20" customHeight="1">
       <c r="A59" s="11" t="s">
@@ -3108,13 +3114,13 @@
       </c>
       <c r="D59" s="11"/>
       <c r="E59" s="11"/>
-      <c r="F59" s="43"/>
-      <c r="G59" s="43"/>
-      <c r="H59" s="43"/>
-      <c r="I59" s="43"/>
-      <c r="J59" s="43"/>
-      <c r="K59" s="43"/>
-      <c r="L59" s="43"/>
+      <c r="F59" s="25"/>
+      <c r="G59" s="25"/>
+      <c r="H59" s="25"/>
+      <c r="I59" s="25"/>
+      <c r="J59" s="25"/>
+      <c r="K59" s="25"/>
+      <c r="L59" s="25"/>
     </row>
     <row r="60" spans="1:12" ht="24" customHeight="1">
       <c r="A60" s="11" t="s">
@@ -3152,15 +3158,15 @@
       </c>
       <c r="D61" s="11"/>
       <c r="E61" s="11"/>
-      <c r="F61" s="23" t="s">
+      <c r="F61" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="G61" s="23"/>
-      <c r="H61" s="23"/>
-      <c r="I61" s="23"/>
-      <c r="J61" s="23"/>
-      <c r="K61" s="23"/>
-      <c r="L61" s="23"/>
+      <c r="G61" s="26"/>
+      <c r="H61" s="26"/>
+      <c r="I61" s="26"/>
+      <c r="J61" s="26"/>
+      <c r="K61" s="26"/>
+      <c r="L61" s="26"/>
     </row>
     <row r="62" spans="1:12" ht="20" customHeight="1">
       <c r="A62" s="11" t="s">
@@ -3176,13 +3182,13 @@
       </c>
       <c r="D62" s="11"/>
       <c r="E62" s="11"/>
-      <c r="F62" s="23"/>
-      <c r="G62" s="23"/>
-      <c r="H62" s="23"/>
-      <c r="I62" s="23"/>
-      <c r="J62" s="23"/>
-      <c r="K62" s="23"/>
-      <c r="L62" s="23"/>
+      <c r="F62" s="26"/>
+      <c r="G62" s="26"/>
+      <c r="H62" s="26"/>
+      <c r="I62" s="26"/>
+      <c r="J62" s="26"/>
+      <c r="K62" s="26"/>
+      <c r="L62" s="26"/>
     </row>
     <row r="63" spans="1:12" ht="24" customHeight="1">
       <c r="A63" s="11" t="s">
@@ -3212,23 +3218,23 @@
       </c>
       <c r="B64" s="11">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$C$7:$C$306,A64)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" s="13">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="D64" s="11"/>
       <c r="E64" s="11"/>
-      <c r="F64" s="44" t="s">
+      <c r="F64" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="G64" s="44"/>
-      <c r="H64" s="44"/>
-      <c r="I64" s="44"/>
-      <c r="J64" s="44"/>
-      <c r="K64" s="44"/>
-      <c r="L64" s="44"/>
+      <c r="G64" s="27"/>
+      <c r="H64" s="27"/>
+      <c r="I64" s="27"/>
+      <c r="J64" s="27"/>
+      <c r="K64" s="27"/>
+      <c r="L64" s="27"/>
     </row>
     <row r="65" spans="1:12" ht="20" customHeight="1">
       <c r="A65" s="11"/>
@@ -3236,13 +3242,13 @@
       <c r="C65" s="11"/>
       <c r="D65" s="11"/>
       <c r="E65" s="11"/>
-      <c r="F65" s="44"/>
-      <c r="G65" s="44"/>
-      <c r="H65" s="44"/>
-      <c r="I65" s="44"/>
-      <c r="J65" s="44"/>
-      <c r="K65" s="44"/>
-      <c r="L65" s="44"/>
+      <c r="F65" s="27"/>
+      <c r="G65" s="27"/>
+      <c r="H65" s="27"/>
+      <c r="I65" s="27"/>
+      <c r="J65" s="27"/>
+      <c r="K65" s="27"/>
+      <c r="L65" s="27"/>
     </row>
     <row r="66" spans="1:12" ht="14.5">
       <c r="A66" s="11"/>
@@ -3274,16 +3280,17 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="F52:L53"/>
-    <mergeCell ref="F55:L56"/>
-    <mergeCell ref="F58:L59"/>
-    <mergeCell ref="F61:L62"/>
-    <mergeCell ref="F64:L65"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="G28:L28"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="F47:L47"/>
-    <mergeCell ref="F49:L50"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C9"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="D7:F9"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="G7:I9"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L9"/>
     <mergeCell ref="J11:L11"/>
     <mergeCell ref="J12:L14"/>
     <mergeCell ref="A16:D16"/>
@@ -3295,17 +3302,16 @@
     <mergeCell ref="D12:F14"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="G12:I14"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C9"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="D7:F9"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I9"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L9"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="G28:L28"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="F47:L47"/>
+    <mergeCell ref="F49:L50"/>
+    <mergeCell ref="F52:L53"/>
+    <mergeCell ref="F55:L56"/>
+    <mergeCell ref="F58:L59"/>
+    <mergeCell ref="F61:L62"/>
+    <mergeCell ref="F64:L65"/>
   </mergeCells>
   <conditionalFormatting sqref="A18:A26">
     <cfRule type="expression" dxfId="19" priority="4">
@@ -3489,118 +3495,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="21"/>
-      <c r="T1" s="21"/>
-      <c r="U1" s="21"/>
-      <c r="V1" s="21"/>
-      <c r="W1" s="21"/>
-      <c r="X1" s="21"/>
-      <c r="Y1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
     </row>
     <row r="2" spans="1:25" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
-      <c r="Y2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
+      <c r="Y2" s="22"/>
     </row>
     <row r="3" spans="1:25" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="23"/>
+      <c r="U3" s="23"/>
+      <c r="V3" s="23"/>
+      <c r="W3" s="23"/>
+      <c r="X3" s="23"/>
+      <c r="Y3" s="23"/>
     </row>
     <row r="4" spans="1:25" ht="30" customHeight="1">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
-      <c r="J4" s="45"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="45"/>
-      <c r="O4" s="45"/>
-      <c r="P4" s="45"/>
-      <c r="Q4" s="45"/>
-      <c r="R4" s="45"/>
-      <c r="S4" s="45"/>
-      <c r="T4" s="45"/>
-      <c r="U4" s="45"/>
-      <c r="V4" s="45"/>
-      <c r="W4" s="45"/>
-      <c r="X4" s="45"/>
-      <c r="Y4" s="45"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+      <c r="W4" s="24"/>
+      <c r="X4" s="24"/>
+      <c r="Y4" s="24"/>
     </row>
     <row r="6" spans="1:25" ht="39" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -3719,11 +3725,11 @@
       <c r="O7" s="5"/>
       <c r="P7" s="7">
         <f t="shared" ref="P7:P70" ca="1" si="0">IF(A7="","",IF(L7="","",MAX(0,IF(O7&lt;&gt;"",O7,TODAY())-L7)))</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q7" s="8" t="str">
         <f t="shared" ref="Q7:Q70" ca="1" si="1">IF(A7="","",IF(OR(G7="Closed",G7="Duplicate",G7="Won't Fix"),"Hoàn tất",IF(M7="","Chưa đặt hạn",IF(TODAY()&gt;M7,"Quá hạn",IF(TODAY()=M7,"Đến hạn","Trong hạn")))))</f>
-        <v>Đến hạn</v>
+        <v>Quá hạn</v>
       </c>
       <c r="R7" s="6"/>
       <c r="S7" s="4" t="s">
@@ -3780,11 +3786,11 @@
       <c r="O8" s="5"/>
       <c r="P8" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="8" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Đến hạn</v>
+        <v>Quá hạn</v>
       </c>
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
@@ -3833,7 +3839,7 @@
       <c r="O9" s="5"/>
       <c r="P9" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q9" s="8" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -3952,7 +3958,7 @@
       <c r="A12" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="21" t="s">
         <v>199</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -4047,14 +4053,30 @@
       <c r="Y13" s="4"/>
     </row>
     <row r="14" spans="1:25" ht="28" customHeight="1">
-      <c r="A14" s="2"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -4068,7 +4090,7 @@
       </c>
       <c r="Q14" s="8" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
+        <v>Chưa đặt hạn</v>
       </c>
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
@@ -12280,7 +12302,7 @@
       <c r="N263" s="5"/>
       <c r="O263" s="5"/>
       <c r="P263" s="7" t="str">
-        <f t="shared" ref="P263:P326" ca="1" si="8">IF(A263="","",IF(L263="","",MAX(0,IF(O263&lt;&gt;"",O263,TODAY())-L263)))</f>
+        <f t="shared" ref="P263:P306" ca="1" si="8">IF(A263="","",IF(L263="","",MAX(0,IF(O263&lt;&gt;"",O263,TODAY())-L263)))</f>
         <v/>
       </c>
       <c r="Q263" s="8" t="str">
@@ -13819,54 +13841,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
     </row>
     <row r="2" spans="1:9" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
     </row>
     <row r="3" spans="1:9" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
     </row>
     <row r="6" spans="1:9" ht="36" customHeight="1">
       <c r="A6" s="9" t="s">
@@ -16141,35 +16163,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:7" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
     </row>
     <row r="4" spans="1:7" ht="29" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -16398,26 +16420,26 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1">
-      <c r="A24" s="47" t="s">
+      <c r="A24" s="48" t="s">
         <v>120</v>
       </c>
-      <c r="B24" s="47"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="47"/>
-      <c r="G24" s="47"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
     </row>
     <row r="26" spans="1:7" ht="29" customHeight="1">
-      <c r="A26" s="48" t="s">
+      <c r="A26" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="48"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -16443,38 +16465,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
     </row>
     <row r="3" spans="1:8" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
     </row>
     <row r="4" spans="1:8" ht="14.5">
       <c r="A4" s="11"/>
@@ -16487,136 +16509,136 @@
       <c r="H4" s="11"/>
     </row>
     <row r="5" spans="1:8" ht="31" customHeight="1">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8" ht="26" customHeight="1">
-      <c r="A6" s="49" t="s">
+      <c r="A6" s="56" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="49"/>
-      <c r="C6" s="50" t="s">
+      <c r="B6" s="56"/>
+      <c r="C6" s="57" t="s">
         <v>126</v>
       </c>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
     </row>
     <row r="7" spans="1:8" ht="26" customHeight="1">
-      <c r="A7" s="49"/>
-      <c r="B7" s="49"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
+      <c r="A7" s="56"/>
+      <c r="B7" s="56"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="57"/>
+      <c r="H7" s="57"/>
     </row>
     <row r="8" spans="1:8" ht="26" customHeight="1">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="56" t="s">
         <v>127</v>
       </c>
-      <c r="B8" s="49"/>
-      <c r="C8" s="51" t="s">
+      <c r="B8" s="56"/>
+      <c r="C8" s="58" t="s">
         <v>128</v>
       </c>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="51"/>
-      <c r="G8" s="51"/>
-      <c r="H8" s="51"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="58"/>
     </row>
     <row r="9" spans="1:8" ht="26" customHeight="1">
-      <c r="A9" s="49"/>
-      <c r="B9" s="49"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
+      <c r="A9" s="56"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="58"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="58"/>
     </row>
     <row r="10" spans="1:8" ht="26" customHeight="1">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="56" t="s">
         <v>129</v>
       </c>
-      <c r="B10" s="49"/>
-      <c r="C10" s="50" t="s">
+      <c r="B10" s="56"/>
+      <c r="C10" s="57" t="s">
         <v>130</v>
       </c>
-      <c r="D10" s="50"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="50"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
+      <c r="H10" s="57"/>
     </row>
     <row r="11" spans="1:8" ht="26" customHeight="1">
-      <c r="A11" s="49"/>
-      <c r="B11" s="49"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
+      <c r="A11" s="56"/>
+      <c r="B11" s="56"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
+      <c r="E11" s="57"/>
+      <c r="F11" s="57"/>
+      <c r="G11" s="57"/>
+      <c r="H11" s="57"/>
     </row>
     <row r="12" spans="1:8" ht="26" customHeight="1">
-      <c r="A12" s="49" t="s">
+      <c r="A12" s="56" t="s">
         <v>131</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="51" t="s">
+      <c r="B12" s="56"/>
+      <c r="C12" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="D12" s="51"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="51"/>
-      <c r="G12" s="51"/>
-      <c r="H12" s="51"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="58"/>
+      <c r="H12" s="58"/>
     </row>
     <row r="13" spans="1:8" ht="26" customHeight="1">
-      <c r="A13" s="49"/>
-      <c r="B13" s="49"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="51"/>
-      <c r="F13" s="51"/>
-      <c r="G13" s="51"/>
-      <c r="H13" s="51"/>
+      <c r="A13" s="56"/>
+      <c r="B13" s="56"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
+      <c r="H13" s="58"/>
     </row>
     <row r="14" spans="1:8" ht="26" customHeight="1">
-      <c r="A14" s="49" t="s">
+      <c r="A14" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="B14" s="49"/>
-      <c r="C14" s="50" t="s">
+      <c r="B14" s="56"/>
+      <c r="C14" s="57" t="s">
         <v>134</v>
       </c>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="50"/>
-      <c r="G14" s="50"/>
-      <c r="H14" s="50"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="57"/>
     </row>
     <row r="15" spans="1:8" ht="26" customHeight="1">
-      <c r="A15" s="49"/>
-      <c r="B15" s="49"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
+      <c r="A15" s="56"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
     </row>
     <row r="16" spans="1:8" ht="14.5">
       <c r="A16" s="11"/>
@@ -16629,16 +16651,16 @@
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="31" customHeight="1">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B17" s="42"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8" ht="26" customHeight="1">
       <c r="A18" s="12" t="s">
@@ -16777,102 +16799,102 @@
       <c r="H24" s="11"/>
     </row>
     <row r="25" spans="1:8" ht="31" customHeight="1">
-      <c r="A25" s="42" t="s">
+      <c r="A25" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="42"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1">
       <c r="A26" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="52" t="s">
+      <c r="B26" s="55" t="s">
         <v>157</v>
       </c>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
       <c r="E26" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="52" t="s">
+      <c r="F26" s="55" t="s">
         <v>158</v>
       </c>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
+      <c r="G26" s="55"/>
+      <c r="H26" s="55"/>
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1">
       <c r="A27" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="52" t="s">
+      <c r="B27" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
       <c r="E27" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="F27" s="52" t="s">
+      <c r="F27" s="55" t="s">
         <v>160</v>
       </c>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="55"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
       <c r="A28" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="52" t="s">
+      <c r="B28" s="55" t="s">
         <v>161</v>
       </c>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
       <c r="E28" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="F28" s="52" t="s">
+      <c r="F28" s="55" t="s">
         <v>162</v>
       </c>
-      <c r="G28" s="52"/>
-      <c r="H28" s="52"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1">
       <c r="A29" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="52" t="s">
+      <c r="B29" s="55" t="s">
         <v>163</v>
       </c>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
       <c r="E29" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="F29" s="52" t="s">
+      <c r="F29" s="55" t="s">
         <v>164</v>
       </c>
-      <c r="G29" s="52"/>
-      <c r="H29" s="52"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="55"/>
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1">
       <c r="A30" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="52" t="s">
+      <c r="B30" s="55" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="52"/>
-      <c r="D30" s="52"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
       <c r="E30" s="20"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="52"/>
-      <c r="H30" s="52"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
     </row>
     <row r="31" spans="1:8" ht="14.5">
       <c r="A31" s="11"/>
@@ -16895,100 +16917,100 @@
       <c r="H32" s="11"/>
     </row>
     <row r="33" spans="1:8" ht="31" customHeight="1">
-      <c r="A33" s="42" t="s">
+      <c r="A33" s="28" t="s">
         <v>166</v>
       </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
     </row>
     <row r="34" spans="1:8" ht="31" customHeight="1">
-      <c r="A34" s="53" t="s">
+      <c r="A34" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="B34" s="53"/>
-      <c r="C34" s="54" t="s">
+      <c r="B34" s="52"/>
+      <c r="C34" s="53" t="s">
         <v>167</v>
       </c>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
+      <c r="D34" s="53"/>
+      <c r="E34" s="53"/>
+      <c r="F34" s="53"/>
+      <c r="G34" s="53"/>
+      <c r="H34" s="53"/>
     </row>
     <row r="35" spans="1:8" ht="31" customHeight="1">
-      <c r="A35" s="53" t="s">
+      <c r="A35" s="52" t="s">
         <v>168</v>
       </c>
-      <c r="B35" s="53"/>
-      <c r="C35" s="55" t="s">
+      <c r="B35" s="52"/>
+      <c r="C35" s="54" t="s">
         <v>169</v>
       </c>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
+      <c r="D35" s="54"/>
+      <c r="E35" s="54"/>
+      <c r="F35" s="54"/>
+      <c r="G35" s="54"/>
+      <c r="H35" s="54"/>
     </row>
     <row r="36" spans="1:8" ht="31" customHeight="1">
-      <c r="A36" s="53" t="s">
+      <c r="A36" s="52" t="s">
         <v>170</v>
       </c>
-      <c r="B36" s="53"/>
-      <c r="C36" s="54" t="s">
+      <c r="B36" s="52"/>
+      <c r="C36" s="53" t="s">
         <v>171</v>
       </c>
-      <c r="D36" s="54"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="54"/>
-      <c r="G36" s="54"/>
-      <c r="H36" s="54"/>
+      <c r="D36" s="53"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="53"/>
+      <c r="G36" s="53"/>
+      <c r="H36" s="53"/>
     </row>
     <row r="37" spans="1:8" ht="31" customHeight="1">
-      <c r="A37" s="53" t="s">
+      <c r="A37" s="52" t="s">
         <v>172</v>
       </c>
-      <c r="B37" s="53"/>
-      <c r="C37" s="55" t="s">
+      <c r="B37" s="52"/>
+      <c r="C37" s="54" t="s">
         <v>173</v>
       </c>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="55"/>
-      <c r="H37" s="55"/>
+      <c r="D37" s="54"/>
+      <c r="E37" s="54"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="54"/>
+      <c r="H37" s="54"/>
     </row>
     <row r="38" spans="1:8" ht="31" customHeight="1">
-      <c r="A38" s="53" t="s">
+      <c r="A38" s="52" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="53"/>
-      <c r="C38" s="54" t="s">
+      <c r="B38" s="52"/>
+      <c r="C38" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="D38" s="54"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
-      <c r="G38" s="54"/>
-      <c r="H38" s="54"/>
+      <c r="D38" s="53"/>
+      <c r="E38" s="53"/>
+      <c r="F38" s="53"/>
+      <c r="G38" s="53"/>
+      <c r="H38" s="53"/>
     </row>
     <row r="39" spans="1:8" ht="31" customHeight="1">
-      <c r="A39" s="53" t="s">
+      <c r="A39" s="52" t="s">
         <v>176</v>
       </c>
-      <c r="B39" s="53"/>
-      <c r="C39" s="55" t="s">
+      <c r="B39" s="52"/>
+      <c r="C39" s="54" t="s">
         <v>177</v>
       </c>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="55"/>
-      <c r="H39" s="55"/>
+      <c r="D39" s="54"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="54"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="54"/>
     </row>
     <row r="40" spans="1:8" ht="14.5">
       <c r="A40" s="11"/>
@@ -17001,76 +17023,76 @@
       <c r="H40" s="11"/>
     </row>
     <row r="41" spans="1:8" ht="31" customHeight="1">
-      <c r="A41" s="42" t="s">
+      <c r="A41" s="28" t="s">
         <v>178</v>
       </c>
-      <c r="B41" s="42"/>
-      <c r="C41" s="42"/>
-      <c r="D41" s="42"/>
-      <c r="E41" s="42"/>
-      <c r="F41" s="42"/>
-      <c r="G41" s="42"/>
-      <c r="H41" s="42"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="28"/>
     </row>
     <row r="42" spans="1:8" ht="29" customHeight="1">
-      <c r="A42" s="56" t="s">
+      <c r="A42" s="50" t="s">
         <v>179</v>
       </c>
-      <c r="B42" s="56"/>
-      <c r="C42" s="56"/>
-      <c r="D42" s="56"/>
-      <c r="E42" s="56"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="56"/>
-      <c r="H42" s="56"/>
+      <c r="B42" s="50"/>
+      <c r="C42" s="50"/>
+      <c r="D42" s="50"/>
+      <c r="E42" s="50"/>
+      <c r="F42" s="50"/>
+      <c r="G42" s="50"/>
+      <c r="H42" s="50"/>
     </row>
     <row r="43" spans="1:8" ht="29" customHeight="1">
-      <c r="A43" s="57" t="s">
+      <c r="A43" s="51" t="s">
         <v>180</v>
       </c>
-      <c r="B43" s="57"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
+      <c r="B43" s="51"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="51"/>
+      <c r="E43" s="51"/>
+      <c r="F43" s="51"/>
+      <c r="G43" s="51"/>
+      <c r="H43" s="51"/>
     </row>
     <row r="44" spans="1:8" ht="29" customHeight="1">
-      <c r="A44" s="56" t="s">
+      <c r="A44" s="50" t="s">
         <v>181</v>
       </c>
-      <c r="B44" s="56"/>
-      <c r="C44" s="56"/>
-      <c r="D44" s="56"/>
-      <c r="E44" s="56"/>
-      <c r="F44" s="56"/>
-      <c r="G44" s="56"/>
-      <c r="H44" s="56"/>
+      <c r="B44" s="50"/>
+      <c r="C44" s="50"/>
+      <c r="D44" s="50"/>
+      <c r="E44" s="50"/>
+      <c r="F44" s="50"/>
+      <c r="G44" s="50"/>
+      <c r="H44" s="50"/>
     </row>
     <row r="45" spans="1:8" ht="29" customHeight="1">
-      <c r="A45" s="57" t="s">
+      <c r="A45" s="51" t="s">
         <v>182</v>
       </c>
-      <c r="B45" s="57"/>
-      <c r="C45" s="57"/>
-      <c r="D45" s="57"/>
-      <c r="E45" s="57"/>
-      <c r="F45" s="57"/>
-      <c r="G45" s="57"/>
-      <c r="H45" s="57"/>
+      <c r="B45" s="51"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="51"/>
+      <c r="E45" s="51"/>
+      <c r="F45" s="51"/>
+      <c r="G45" s="51"/>
+      <c r="H45" s="51"/>
     </row>
     <row r="46" spans="1:8" ht="29" customHeight="1">
-      <c r="A46" s="56" t="s">
+      <c r="A46" s="50" t="s">
         <v>183</v>
       </c>
-      <c r="B46" s="56"/>
-      <c r="C46" s="56"/>
-      <c r="D46" s="56"/>
-      <c r="E46" s="56"/>
-      <c r="F46" s="56"/>
-      <c r="G46" s="56"/>
-      <c r="H46" s="56"/>
+      <c r="B46" s="50"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="50"/>
+      <c r="E46" s="50"/>
+      <c r="F46" s="50"/>
+      <c r="G46" s="50"/>
+      <c r="H46" s="50"/>
     </row>
     <row r="47" spans="1:8" ht="14.5">
       <c r="A47" s="11"/>
@@ -17084,50 +17106,50 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="A42:H42"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="C6:H7"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:H9"/>
+    <mergeCell ref="A10:B11"/>
+    <mergeCell ref="C10:H11"/>
+    <mergeCell ref="A12:B13"/>
+    <mergeCell ref="C12:H13"/>
+    <mergeCell ref="A14:B15"/>
+    <mergeCell ref="C14:H15"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:H34"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="C35:H35"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="C36:H36"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="C37:H37"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="A33:H33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="A14:B15"/>
-    <mergeCell ref="C14:H15"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:H9"/>
-    <mergeCell ref="A10:B11"/>
-    <mergeCell ref="C10:H11"/>
-    <mergeCell ref="A12:B13"/>
-    <mergeCell ref="C12:H13"/>
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="C6:H7"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A46:H46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Feature/update UI authen (#101)
* review talent candidate

* fix sidebar

* fix all sidebar

* ui v2

* fe v2

* ui admin v3

* review v1

* fix bug update department
</commit_message>
<xml_diff>
--- a/docs/members/linhdn/Professional_Bug_Tracker_Template.xlsx
+++ b/docs/members/linhdn/Professional_Bug_Tracker_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dowload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KÌ 5\SWP\hireflow-api\RetireManagement\SWP_RMS_Group-2\docs\members\linhdn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72C1335-D8F0-4F5B-AAB1-0A6209F55F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBFDBA3-7340-468B-A972-48500F2FEC75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="204">
   <si>
     <t>BUG QUALITY DASHBOARD</t>
   </si>
@@ -644,6 +644,12 @@
   </si>
   <si>
     <t>Lỗi FE khi bấm đóng dợt tuyể</t>
+  </si>
+  <si>
+    <t>B07</t>
+  </si>
+  <si>
+    <t>lỗi  mất kết nối sever</t>
   </si>
 </sst>
 </file>
@@ -944,14 +950,59 @@
     <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -977,61 +1028,13 @@
     <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1041,13 +1044,16 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1344,7 +1350,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2</c:v>
@@ -1520,7 +1526,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2</c:v>
@@ -1967,66 +1973,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
     </row>
     <row r="2" spans="1:12" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
     </row>
     <row r="3" spans="1:12" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
     </row>
     <row r="4" spans="1:12" ht="28" customHeight="1">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
     </row>
     <row r="5" spans="1:12" ht="14.5">
       <c r="A5" s="11"/>
@@ -2043,80 +2049,80 @@
       <c r="L5" s="11"/>
     </row>
     <row r="6" spans="1:12" ht="29" customHeight="1">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="26" t="s">
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="28" t="s">
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="30" t="s">
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="30"/>
-      <c r="L6" s="30"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="45"/>
     </row>
     <row r="7" spans="1:12" ht="24" customHeight="1">
-      <c r="A7" s="25">
+      <c r="A7" s="40">
         <f>COUNTIF('Bug Log'!$A$7:$A$306,"&lt;&gt;")</f>
-        <v>7</v>
-      </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="27">
+        <v>8</v>
+      </c>
+      <c r="B7" s="40"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="42">
         <f>COUNTIF('Bug Log'!$A$7:$A$306,"&lt;&gt;")-COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Closed")-COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Duplicate")-COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Won't Fix")</f>
-        <v>7</v>
-      </c>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="29">
+        <v>8</v>
+      </c>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="44">
         <f ca="1">COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$Q$7:$Q$306,"Quá hạn")</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="31">
+        <v>2</v>
+      </c>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="46">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,"Closed")</f>
         <v>0</v>
       </c>
-      <c r="K7" s="31"/>
-      <c r="L7" s="31"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
     </row>
     <row r="8" spans="1:12" ht="24" customHeight="1">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="31"/>
+      <c r="A8" s="40"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="46"/>
+      <c r="K8" s="46"/>
+      <c r="L8" s="46"/>
     </row>
     <row r="9" spans="1:12" ht="24" customHeight="1">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
+      <c r="A9" s="40"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="46"/>
+      <c r="K9" s="46"/>
+      <c r="L9" s="46"/>
     </row>
     <row r="10" spans="1:12" ht="14.5">
       <c r="A10" s="11"/>
@@ -2148,16 +2154,16 @@
       </c>
       <c r="H11" s="36"/>
       <c r="I11" s="36"/>
-      <c r="J11" s="39" t="s">
+      <c r="J11" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="K11" s="39"/>
-      <c r="L11" s="39"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
     </row>
     <row r="12" spans="1:12" ht="24" customHeight="1">
       <c r="A12" s="33">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$E$7:$E$306,"Blocker")+COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$E$7:$E$306,"Critical")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="33"/>
@@ -2173,12 +2179,12 @@
       </c>
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
-      <c r="J12" s="40">
+      <c r="J12" s="30">
         <f ca="1">IFERROR(AVERAGE('Bug Log'!$P$7:$P$306),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
+        <v>7</v>
+      </c>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
     </row>
     <row r="13" spans="1:12" ht="24" customHeight="1">
       <c r="A13" s="33"/>
@@ -2190,9 +2196,9 @@
       <c r="G13" s="38"/>
       <c r="H13" s="38"/>
       <c r="I13" s="38"/>
-      <c r="J13" s="41"/>
-      <c r="K13" s="41"/>
-      <c r="L13" s="41"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
     </row>
     <row r="14" spans="1:12" ht="24" customHeight="1">
       <c r="A14" s="33"/>
@@ -2204,9 +2210,9 @@
       <c r="G14" s="38"/>
       <c r="H14" s="38"/>
       <c r="I14" s="38"/>
-      <c r="J14" s="41"/>
-      <c r="K14" s="41"/>
-      <c r="L14" s="41"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
     </row>
     <row r="15" spans="1:12" ht="14.5">
       <c r="A15" s="11"/>
@@ -2223,24 +2229,24 @@
       <c r="L15" s="11"/>
     </row>
     <row r="16" spans="1:12" ht="31" customHeight="1">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
       <c r="E16" s="11"/>
-      <c r="F16" s="42" t="s">
+      <c r="F16" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42" t="s">
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="K16" s="42"/>
-      <c r="L16" s="42"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="28"/>
     </row>
     <row r="17" spans="1:12" ht="25" customHeight="1">
       <c r="A17" s="12" t="s">
@@ -2280,11 +2286,11 @@
       </c>
       <c r="B18" s="14">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$G$7:$G$306,A18)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" s="15">
         <f t="shared" ref="C18:C26" si="0">IFERROR(B18/$A$7,0)</f>
-        <v>0.7142857142857143</v>
+        <v>0.75</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
@@ -2293,11 +2299,11 @@
       </c>
       <c r="G18" s="11">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$E$7:$E$306,F18)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="13">
         <f>IFERROR(G18/$A$7,0)</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I18" s="11"/>
       <c r="J18" s="11" t="s">
@@ -2305,11 +2311,11 @@
       </c>
       <c r="K18" s="11">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$F$7:$F$306,J18)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" s="13">
         <f>IFERROR(K18/$A$7,0)</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="25" customHeight="1">
@@ -2322,7 +2328,7 @@
       </c>
       <c r="C19" s="15">
         <f t="shared" si="0"/>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
@@ -2335,7 +2341,7 @@
       </c>
       <c r="H19" s="13">
         <f>IFERROR(G19/$A$7,0)</f>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
       <c r="I19" s="11"/>
       <c r="J19" s="11" t="s">
@@ -2347,7 +2353,7 @@
       </c>
       <c r="L19" s="13">
         <f>IFERROR(K19/$A$7,0)</f>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="25" customHeight="1">
@@ -2373,7 +2379,7 @@
       </c>
       <c r="H20" s="13">
         <f>IFERROR(G20/$A$7,0)</f>
-        <v>0.14285714285714285</v>
+        <v>0.125</v>
       </c>
       <c r="I20" s="11"/>
       <c r="J20" s="11" t="s">
@@ -2385,7 +2391,7 @@
       </c>
       <c r="L20" s="13">
         <f>IFERROR(K20/$A$7,0)</f>
-        <v>0.42857142857142855</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="25" customHeight="1">
@@ -2411,7 +2417,7 @@
       </c>
       <c r="H21" s="13">
         <f>IFERROR(G21/$A$7,0)</f>
-        <v>0.5714285714285714</v>
+        <v>0.5</v>
       </c>
       <c r="I21" s="11"/>
       <c r="J21" s="11" t="s">
@@ -2423,7 +2429,7 @@
       </c>
       <c r="L21" s="13">
         <f>IFERROR(K21/$A$7,0)</f>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="25" customHeight="1">
@@ -2559,22 +2565,22 @@
       <c r="L27" s="11"/>
     </row>
     <row r="28" spans="1:12" ht="31" customHeight="1">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42" t="s">
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="H28" s="42"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="42"/>
-      <c r="K28" s="42"/>
-      <c r="L28" s="42"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="28"/>
     </row>
     <row r="29" spans="1:12" ht="14.5">
       <c r="A29" s="11"/>
@@ -2829,22 +2835,22 @@
       <c r="L46" s="11"/>
     </row>
     <row r="47" spans="1:12" ht="31" customHeight="1">
-      <c r="A47" s="42" t="s">
+      <c r="A47" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="B47" s="42"/>
-      <c r="C47" s="42"/>
-      <c r="D47" s="42"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
       <c r="E47" s="11"/>
-      <c r="F47" s="42" t="s">
+      <c r="F47" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="G47" s="42"/>
-      <c r="H47" s="42"/>
-      <c r="I47" s="42"/>
-      <c r="J47" s="42"/>
-      <c r="K47" s="42"/>
-      <c r="L47" s="42"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="28"/>
+      <c r="I47" s="28"/>
+      <c r="J47" s="28"/>
+      <c r="K47" s="28"/>
+      <c r="L47" s="28"/>
     </row>
     <row r="48" spans="1:12" ht="27" customHeight="1">
       <c r="A48" s="12" t="s">
@@ -2880,15 +2886,15 @@
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="11"/>
-      <c r="F49" s="23" t="s">
+      <c r="F49" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="G49" s="23"/>
-      <c r="H49" s="23"/>
-      <c r="I49" s="23"/>
-      <c r="J49" s="23"/>
-      <c r="K49" s="23"/>
-      <c r="L49" s="23"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="26"/>
+      <c r="I49" s="26"/>
+      <c r="J49" s="26"/>
+      <c r="K49" s="26"/>
+      <c r="L49" s="26"/>
     </row>
     <row r="50" spans="1:12" ht="20" customHeight="1">
       <c r="A50" s="11" t="s">
@@ -2904,13 +2910,13 @@
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="11"/>
-      <c r="F50" s="23"/>
-      <c r="G50" s="23"/>
-      <c r="H50" s="23"/>
-      <c r="I50" s="23"/>
-      <c r="J50" s="23"/>
-      <c r="K50" s="23"/>
-      <c r="L50" s="23"/>
+      <c r="F50" s="26"/>
+      <c r="G50" s="26"/>
+      <c r="H50" s="26"/>
+      <c r="I50" s="26"/>
+      <c r="J50" s="26"/>
+      <c r="K50" s="26"/>
+      <c r="L50" s="26"/>
     </row>
     <row r="51" spans="1:12" ht="24" customHeight="1">
       <c r="A51" s="11" t="s">
@@ -2922,7 +2928,7 @@
       </c>
       <c r="C51" s="13">
         <f t="shared" si="1"/>
-        <v>0.14285714285714285</v>
+        <v>0.125</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="11"/>
@@ -2948,15 +2954,15 @@
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="11"/>
-      <c r="F52" s="43" t="s">
+      <c r="F52" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="G52" s="43"/>
-      <c r="H52" s="43"/>
-      <c r="I52" s="43"/>
-      <c r="J52" s="43"/>
-      <c r="K52" s="43"/>
-      <c r="L52" s="43"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="25"/>
+      <c r="I52" s="25"/>
+      <c r="J52" s="25"/>
+      <c r="K52" s="25"/>
+      <c r="L52" s="25"/>
     </row>
     <row r="53" spans="1:12" ht="20" customHeight="1">
       <c r="A53" s="11" t="s">
@@ -2972,13 +2978,13 @@
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="11"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="43"/>
-      <c r="I53" s="43"/>
-      <c r="J53" s="43"/>
-      <c r="K53" s="43"/>
-      <c r="L53" s="43"/>
+      <c r="F53" s="25"/>
+      <c r="G53" s="25"/>
+      <c r="H53" s="25"/>
+      <c r="I53" s="25"/>
+      <c r="J53" s="25"/>
+      <c r="K53" s="25"/>
+      <c r="L53" s="25"/>
     </row>
     <row r="54" spans="1:12" ht="24" customHeight="1">
       <c r="A54" s="11" t="s">
@@ -2990,7 +2996,7 @@
       </c>
       <c r="C54" s="13">
         <f t="shared" si="1"/>
-        <v>0.2857142857142857</v>
+        <v>0.25</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="11"/>
@@ -3012,19 +3018,19 @@
       </c>
       <c r="C55" s="13">
         <f t="shared" si="1"/>
-        <v>0.42857142857142855</v>
+        <v>0.375</v>
       </c>
       <c r="D55" s="11"/>
       <c r="E55" s="11"/>
-      <c r="F55" s="23" t="s">
+      <c r="F55" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="G55" s="23"/>
-      <c r="H55" s="23"/>
-      <c r="I55" s="23"/>
-      <c r="J55" s="23"/>
-      <c r="K55" s="23"/>
-      <c r="L55" s="23"/>
+      <c r="G55" s="26"/>
+      <c r="H55" s="26"/>
+      <c r="I55" s="26"/>
+      <c r="J55" s="26"/>
+      <c r="K55" s="26"/>
+      <c r="L55" s="26"/>
     </row>
     <row r="56" spans="1:12" ht="20" customHeight="1">
       <c r="A56" s="11" t="s">
@@ -3040,13 +3046,13 @@
       </c>
       <c r="D56" s="11"/>
       <c r="E56" s="11"/>
-      <c r="F56" s="23"/>
-      <c r="G56" s="23"/>
-      <c r="H56" s="23"/>
-      <c r="I56" s="23"/>
-      <c r="J56" s="23"/>
-      <c r="K56" s="23"/>
-      <c r="L56" s="23"/>
+      <c r="F56" s="26"/>
+      <c r="G56" s="26"/>
+      <c r="H56" s="26"/>
+      <c r="I56" s="26"/>
+      <c r="J56" s="26"/>
+      <c r="K56" s="26"/>
+      <c r="L56" s="26"/>
     </row>
     <row r="57" spans="1:12" ht="24" customHeight="1">
       <c r="A57" s="11" t="s">
@@ -3058,7 +3064,7 @@
       </c>
       <c r="C57" s="13">
         <f t="shared" si="1"/>
-        <v>0.14285714285714285</v>
+        <v>0.125</v>
       </c>
       <c r="D57" s="11"/>
       <c r="E57" s="11"/>
@@ -3084,15 +3090,15 @@
       </c>
       <c r="D58" s="11"/>
       <c r="E58" s="11"/>
-      <c r="F58" s="43" t="s">
+      <c r="F58" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="G58" s="43"/>
-      <c r="H58" s="43"/>
-      <c r="I58" s="43"/>
-      <c r="J58" s="43"/>
-      <c r="K58" s="43"/>
-      <c r="L58" s="43"/>
+      <c r="G58" s="25"/>
+      <c r="H58" s="25"/>
+      <c r="I58" s="25"/>
+      <c r="J58" s="25"/>
+      <c r="K58" s="25"/>
+      <c r="L58" s="25"/>
     </row>
     <row r="59" spans="1:12" ht="20" customHeight="1">
       <c r="A59" s="11" t="s">
@@ -3108,13 +3114,13 @@
       </c>
       <c r="D59" s="11"/>
       <c r="E59" s="11"/>
-      <c r="F59" s="43"/>
-      <c r="G59" s="43"/>
-      <c r="H59" s="43"/>
-      <c r="I59" s="43"/>
-      <c r="J59" s="43"/>
-      <c r="K59" s="43"/>
-      <c r="L59" s="43"/>
+      <c r="F59" s="25"/>
+      <c r="G59" s="25"/>
+      <c r="H59" s="25"/>
+      <c r="I59" s="25"/>
+      <c r="J59" s="25"/>
+      <c r="K59" s="25"/>
+      <c r="L59" s="25"/>
     </row>
     <row r="60" spans="1:12" ht="24" customHeight="1">
       <c r="A60" s="11" t="s">
@@ -3152,15 +3158,15 @@
       </c>
       <c r="D61" s="11"/>
       <c r="E61" s="11"/>
-      <c r="F61" s="23" t="s">
+      <c r="F61" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="G61" s="23"/>
-      <c r="H61" s="23"/>
-      <c r="I61" s="23"/>
-      <c r="J61" s="23"/>
-      <c r="K61" s="23"/>
-      <c r="L61" s="23"/>
+      <c r="G61" s="26"/>
+      <c r="H61" s="26"/>
+      <c r="I61" s="26"/>
+      <c r="J61" s="26"/>
+      <c r="K61" s="26"/>
+      <c r="L61" s="26"/>
     </row>
     <row r="62" spans="1:12" ht="20" customHeight="1">
       <c r="A62" s="11" t="s">
@@ -3176,13 +3182,13 @@
       </c>
       <c r="D62" s="11"/>
       <c r="E62" s="11"/>
-      <c r="F62" s="23"/>
-      <c r="G62" s="23"/>
-      <c r="H62" s="23"/>
-      <c r="I62" s="23"/>
-      <c r="J62" s="23"/>
-      <c r="K62" s="23"/>
-      <c r="L62" s="23"/>
+      <c r="F62" s="26"/>
+      <c r="G62" s="26"/>
+      <c r="H62" s="26"/>
+      <c r="I62" s="26"/>
+      <c r="J62" s="26"/>
+      <c r="K62" s="26"/>
+      <c r="L62" s="26"/>
     </row>
     <row r="63" spans="1:12" ht="24" customHeight="1">
       <c r="A63" s="11" t="s">
@@ -3212,23 +3218,23 @@
       </c>
       <c r="B64" s="11">
         <f>COUNTIFS('Bug Log'!$A$7:$A$306,"&lt;&gt;",'Bug Log'!$C$7:$C$306,A64)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C64" s="13">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="D64" s="11"/>
       <c r="E64" s="11"/>
-      <c r="F64" s="44" t="s">
+      <c r="F64" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="G64" s="44"/>
-      <c r="H64" s="44"/>
-      <c r="I64" s="44"/>
-      <c r="J64" s="44"/>
-      <c r="K64" s="44"/>
-      <c r="L64" s="44"/>
+      <c r="G64" s="27"/>
+      <c r="H64" s="27"/>
+      <c r="I64" s="27"/>
+      <c r="J64" s="27"/>
+      <c r="K64" s="27"/>
+      <c r="L64" s="27"/>
     </row>
     <row r="65" spans="1:12" ht="20" customHeight="1">
       <c r="A65" s="11"/>
@@ -3236,13 +3242,13 @@
       <c r="C65" s="11"/>
       <c r="D65" s="11"/>
       <c r="E65" s="11"/>
-      <c r="F65" s="44"/>
-      <c r="G65" s="44"/>
-      <c r="H65" s="44"/>
-      <c r="I65" s="44"/>
-      <c r="J65" s="44"/>
-      <c r="K65" s="44"/>
-      <c r="L65" s="44"/>
+      <c r="F65" s="27"/>
+      <c r="G65" s="27"/>
+      <c r="H65" s="27"/>
+      <c r="I65" s="27"/>
+      <c r="J65" s="27"/>
+      <c r="K65" s="27"/>
+      <c r="L65" s="27"/>
     </row>
     <row r="66" spans="1:12" ht="14.5">
       <c r="A66" s="11"/>
@@ -3274,16 +3280,17 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="F52:L53"/>
-    <mergeCell ref="F55:L56"/>
-    <mergeCell ref="F58:L59"/>
-    <mergeCell ref="F61:L62"/>
-    <mergeCell ref="F64:L65"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="G28:L28"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="F47:L47"/>
-    <mergeCell ref="F49:L50"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C9"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="D7:F9"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="G7:I9"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L9"/>
     <mergeCell ref="J11:L11"/>
     <mergeCell ref="J12:L14"/>
     <mergeCell ref="A16:D16"/>
@@ -3295,17 +3302,16 @@
     <mergeCell ref="D12:F14"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="G12:I14"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C9"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="D7:F9"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I9"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L9"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="G28:L28"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="F47:L47"/>
+    <mergeCell ref="F49:L50"/>
+    <mergeCell ref="F52:L53"/>
+    <mergeCell ref="F55:L56"/>
+    <mergeCell ref="F58:L59"/>
+    <mergeCell ref="F61:L62"/>
+    <mergeCell ref="F64:L65"/>
   </mergeCells>
   <conditionalFormatting sqref="A18:A26">
     <cfRule type="expression" dxfId="19" priority="4">
@@ -3489,118 +3495,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="21"/>
-      <c r="T1" s="21"/>
-      <c r="U1" s="21"/>
-      <c r="V1" s="21"/>
-      <c r="W1" s="21"/>
-      <c r="X1" s="21"/>
-      <c r="Y1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
     </row>
     <row r="2" spans="1:25" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
-      <c r="Y2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
+      <c r="Y2" s="22"/>
     </row>
     <row r="3" spans="1:25" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="23"/>
+      <c r="U3" s="23"/>
+      <c r="V3" s="23"/>
+      <c r="W3" s="23"/>
+      <c r="X3" s="23"/>
+      <c r="Y3" s="23"/>
     </row>
     <row r="4" spans="1:25" ht="30" customHeight="1">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
-      <c r="J4" s="45"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="45"/>
-      <c r="O4" s="45"/>
-      <c r="P4" s="45"/>
-      <c r="Q4" s="45"/>
-      <c r="R4" s="45"/>
-      <c r="S4" s="45"/>
-      <c r="T4" s="45"/>
-      <c r="U4" s="45"/>
-      <c r="V4" s="45"/>
-      <c r="W4" s="45"/>
-      <c r="X4" s="45"/>
-      <c r="Y4" s="45"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+      <c r="W4" s="24"/>
+      <c r="X4" s="24"/>
+      <c r="Y4" s="24"/>
     </row>
     <row r="6" spans="1:25" ht="39" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -3719,11 +3725,11 @@
       <c r="O7" s="5"/>
       <c r="P7" s="7">
         <f t="shared" ref="P7:P70" ca="1" si="0">IF(A7="","",IF(L7="","",MAX(0,IF(O7&lt;&gt;"",O7,TODAY())-L7)))</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q7" s="8" t="str">
         <f t="shared" ref="Q7:Q70" ca="1" si="1">IF(A7="","",IF(OR(G7="Closed",G7="Duplicate",G7="Won't Fix"),"Hoàn tất",IF(M7="","Chưa đặt hạn",IF(TODAY()&gt;M7,"Quá hạn",IF(TODAY()=M7,"Đến hạn","Trong hạn")))))</f>
-        <v>Đến hạn</v>
+        <v>Quá hạn</v>
       </c>
       <c r="R7" s="6"/>
       <c r="S7" s="4" t="s">
@@ -3780,11 +3786,11 @@
       <c r="O8" s="5"/>
       <c r="P8" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="8" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>Đến hạn</v>
+        <v>Quá hạn</v>
       </c>
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
@@ -3833,7 +3839,7 @@
       <c r="O9" s="5"/>
       <c r="P9" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q9" s="8" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -3952,7 +3958,7 @@
       <c r="A12" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="21" t="s">
         <v>199</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -4047,14 +4053,30 @@
       <c r="Y13" s="4"/>
     </row>
     <row r="14" spans="1:25" ht="28" customHeight="1">
-      <c r="A14" s="2"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -4068,7 +4090,7 @@
       </c>
       <c r="Q14" s="8" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
+        <v>Chưa đặt hạn</v>
       </c>
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
@@ -12280,7 +12302,7 @@
       <c r="N263" s="5"/>
       <c r="O263" s="5"/>
       <c r="P263" s="7" t="str">
-        <f t="shared" ref="P263:P326" ca="1" si="8">IF(A263="","",IF(L263="","",MAX(0,IF(O263&lt;&gt;"",O263,TODAY())-L263)))</f>
+        <f t="shared" ref="P263:P306" ca="1" si="8">IF(A263="","",IF(L263="","",MAX(0,IF(O263&lt;&gt;"",O263,TODAY())-L263)))</f>
         <v/>
       </c>
       <c r="Q263" s="8" t="str">
@@ -13819,54 +13841,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
     </row>
     <row r="2" spans="1:9" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
     </row>
     <row r="3" spans="1:9" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
     </row>
     <row r="6" spans="1:9" ht="36" customHeight="1">
       <c r="A6" s="9" t="s">
@@ -16141,35 +16163,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:7" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
     </row>
     <row r="4" spans="1:7" ht="29" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -16398,26 +16420,26 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1">
-      <c r="A24" s="47" t="s">
+      <c r="A24" s="48" t="s">
         <v>120</v>
       </c>
-      <c r="B24" s="47"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="47"/>
-      <c r="G24" s="47"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
     </row>
     <row r="26" spans="1:7" ht="29" customHeight="1">
-      <c r="A26" s="48" t="s">
+      <c r="A26" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="48"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -16443,38 +16465,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25" customHeight="1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="25" customHeight="1">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
     </row>
     <row r="3" spans="1:8" ht="27" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
     </row>
     <row r="4" spans="1:8" ht="14.5">
       <c r="A4" s="11"/>
@@ -16487,136 +16509,136 @@
       <c r="H4" s="11"/>
     </row>
     <row r="5" spans="1:8" ht="31" customHeight="1">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8" ht="26" customHeight="1">
-      <c r="A6" s="49" t="s">
+      <c r="A6" s="56" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="49"/>
-      <c r="C6" s="50" t="s">
+      <c r="B6" s="56"/>
+      <c r="C6" s="57" t="s">
         <v>126</v>
       </c>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
     </row>
     <row r="7" spans="1:8" ht="26" customHeight="1">
-      <c r="A7" s="49"/>
-      <c r="B7" s="49"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
+      <c r="A7" s="56"/>
+      <c r="B7" s="56"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="57"/>
+      <c r="H7" s="57"/>
     </row>
     <row r="8" spans="1:8" ht="26" customHeight="1">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="56" t="s">
         <v>127</v>
       </c>
-      <c r="B8" s="49"/>
-      <c r="C8" s="51" t="s">
+      <c r="B8" s="56"/>
+      <c r="C8" s="58" t="s">
         <v>128</v>
       </c>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="51"/>
-      <c r="G8" s="51"/>
-      <c r="H8" s="51"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="58"/>
     </row>
     <row r="9" spans="1:8" ht="26" customHeight="1">
-      <c r="A9" s="49"/>
-      <c r="B9" s="49"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
+      <c r="A9" s="56"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="58"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="58"/>
     </row>
     <row r="10" spans="1:8" ht="26" customHeight="1">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="56" t="s">
         <v>129</v>
       </c>
-      <c r="B10" s="49"/>
-      <c r="C10" s="50" t="s">
+      <c r="B10" s="56"/>
+      <c r="C10" s="57" t="s">
         <v>130</v>
       </c>
-      <c r="D10" s="50"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="50"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
+      <c r="H10" s="57"/>
     </row>
     <row r="11" spans="1:8" ht="26" customHeight="1">
-      <c r="A11" s="49"/>
-      <c r="B11" s="49"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
+      <c r="A11" s="56"/>
+      <c r="B11" s="56"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
+      <c r="E11" s="57"/>
+      <c r="F11" s="57"/>
+      <c r="G11" s="57"/>
+      <c r="H11" s="57"/>
     </row>
     <row r="12" spans="1:8" ht="26" customHeight="1">
-      <c r="A12" s="49" t="s">
+      <c r="A12" s="56" t="s">
         <v>131</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="51" t="s">
+      <c r="B12" s="56"/>
+      <c r="C12" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="D12" s="51"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="51"/>
-      <c r="G12" s="51"/>
-      <c r="H12" s="51"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="58"/>
+      <c r="H12" s="58"/>
     </row>
     <row r="13" spans="1:8" ht="26" customHeight="1">
-      <c r="A13" s="49"/>
-      <c r="B13" s="49"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="51"/>
-      <c r="F13" s="51"/>
-      <c r="G13" s="51"/>
-      <c r="H13" s="51"/>
+      <c r="A13" s="56"/>
+      <c r="B13" s="56"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
+      <c r="H13" s="58"/>
     </row>
     <row r="14" spans="1:8" ht="26" customHeight="1">
-      <c r="A14" s="49" t="s">
+      <c r="A14" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="B14" s="49"/>
-      <c r="C14" s="50" t="s">
+      <c r="B14" s="56"/>
+      <c r="C14" s="57" t="s">
         <v>134</v>
       </c>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="50"/>
-      <c r="G14" s="50"/>
-      <c r="H14" s="50"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="57"/>
     </row>
     <row r="15" spans="1:8" ht="26" customHeight="1">
-      <c r="A15" s="49"/>
-      <c r="B15" s="49"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
+      <c r="A15" s="56"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
     </row>
     <row r="16" spans="1:8" ht="14.5">
       <c r="A16" s="11"/>
@@ -16629,16 +16651,16 @@
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="31" customHeight="1">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B17" s="42"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8" ht="26" customHeight="1">
       <c r="A18" s="12" t="s">
@@ -16777,102 +16799,102 @@
       <c r="H24" s="11"/>
     </row>
     <row r="25" spans="1:8" ht="31" customHeight="1">
-      <c r="A25" s="42" t="s">
+      <c r="A25" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="42"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1">
       <c r="A26" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="52" t="s">
+      <c r="B26" s="55" t="s">
         <v>157</v>
       </c>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
       <c r="E26" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="52" t="s">
+      <c r="F26" s="55" t="s">
         <v>158</v>
       </c>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
+      <c r="G26" s="55"/>
+      <c r="H26" s="55"/>
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1">
       <c r="A27" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="52" t="s">
+      <c r="B27" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
       <c r="E27" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="F27" s="52" t="s">
+      <c r="F27" s="55" t="s">
         <v>160</v>
       </c>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="55"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
       <c r="A28" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="52" t="s">
+      <c r="B28" s="55" t="s">
         <v>161</v>
       </c>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
       <c r="E28" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="F28" s="52" t="s">
+      <c r="F28" s="55" t="s">
         <v>162</v>
       </c>
-      <c r="G28" s="52"/>
-      <c r="H28" s="52"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1">
       <c r="A29" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="52" t="s">
+      <c r="B29" s="55" t="s">
         <v>163</v>
       </c>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
       <c r="E29" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="F29" s="52" t="s">
+      <c r="F29" s="55" t="s">
         <v>164</v>
       </c>
-      <c r="G29" s="52"/>
-      <c r="H29" s="52"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="55"/>
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1">
       <c r="A30" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="52" t="s">
+      <c r="B30" s="55" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="52"/>
-      <c r="D30" s="52"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
       <c r="E30" s="20"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="52"/>
-      <c r="H30" s="52"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
     </row>
     <row r="31" spans="1:8" ht="14.5">
       <c r="A31" s="11"/>
@@ -16895,100 +16917,100 @@
       <c r="H32" s="11"/>
     </row>
     <row r="33" spans="1:8" ht="31" customHeight="1">
-      <c r="A33" s="42" t="s">
+      <c r="A33" s="28" t="s">
         <v>166</v>
       </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
     </row>
     <row r="34" spans="1:8" ht="31" customHeight="1">
-      <c r="A34" s="53" t="s">
+      <c r="A34" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="B34" s="53"/>
-      <c r="C34" s="54" t="s">
+      <c r="B34" s="52"/>
+      <c r="C34" s="53" t="s">
         <v>167</v>
       </c>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
+      <c r="D34" s="53"/>
+      <c r="E34" s="53"/>
+      <c r="F34" s="53"/>
+      <c r="G34" s="53"/>
+      <c r="H34" s="53"/>
     </row>
     <row r="35" spans="1:8" ht="31" customHeight="1">
-      <c r="A35" s="53" t="s">
+      <c r="A35" s="52" t="s">
         <v>168</v>
       </c>
-      <c r="B35" s="53"/>
-      <c r="C35" s="55" t="s">
+      <c r="B35" s="52"/>
+      <c r="C35" s="54" t="s">
         <v>169</v>
       </c>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
+      <c r="D35" s="54"/>
+      <c r="E35" s="54"/>
+      <c r="F35" s="54"/>
+      <c r="G35" s="54"/>
+      <c r="H35" s="54"/>
     </row>
     <row r="36" spans="1:8" ht="31" customHeight="1">
-      <c r="A36" s="53" t="s">
+      <c r="A36" s="52" t="s">
         <v>170</v>
       </c>
-      <c r="B36" s="53"/>
-      <c r="C36" s="54" t="s">
+      <c r="B36" s="52"/>
+      <c r="C36" s="53" t="s">
         <v>171</v>
       </c>
-      <c r="D36" s="54"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="54"/>
-      <c r="G36" s="54"/>
-      <c r="H36" s="54"/>
+      <c r="D36" s="53"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="53"/>
+      <c r="G36" s="53"/>
+      <c r="H36" s="53"/>
     </row>
     <row r="37" spans="1:8" ht="31" customHeight="1">
-      <c r="A37" s="53" t="s">
+      <c r="A37" s="52" t="s">
         <v>172</v>
       </c>
-      <c r="B37" s="53"/>
-      <c r="C37" s="55" t="s">
+      <c r="B37" s="52"/>
+      <c r="C37" s="54" t="s">
         <v>173</v>
       </c>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="55"/>
-      <c r="H37" s="55"/>
+      <c r="D37" s="54"/>
+      <c r="E37" s="54"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="54"/>
+      <c r="H37" s="54"/>
     </row>
     <row r="38" spans="1:8" ht="31" customHeight="1">
-      <c r="A38" s="53" t="s">
+      <c r="A38" s="52" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="53"/>
-      <c r="C38" s="54" t="s">
+      <c r="B38" s="52"/>
+      <c r="C38" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="D38" s="54"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
-      <c r="G38" s="54"/>
-      <c r="H38" s="54"/>
+      <c r="D38" s="53"/>
+      <c r="E38" s="53"/>
+      <c r="F38" s="53"/>
+      <c r="G38" s="53"/>
+      <c r="H38" s="53"/>
     </row>
     <row r="39" spans="1:8" ht="31" customHeight="1">
-      <c r="A39" s="53" t="s">
+      <c r="A39" s="52" t="s">
         <v>176</v>
       </c>
-      <c r="B39" s="53"/>
-      <c r="C39" s="55" t="s">
+      <c r="B39" s="52"/>
+      <c r="C39" s="54" t="s">
         <v>177</v>
       </c>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="55"/>
-      <c r="H39" s="55"/>
+      <c r="D39" s="54"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="54"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="54"/>
     </row>
     <row r="40" spans="1:8" ht="14.5">
       <c r="A40" s="11"/>
@@ -17001,76 +17023,76 @@
       <c r="H40" s="11"/>
     </row>
     <row r="41" spans="1:8" ht="31" customHeight="1">
-      <c r="A41" s="42" t="s">
+      <c r="A41" s="28" t="s">
         <v>178</v>
       </c>
-      <c r="B41" s="42"/>
-      <c r="C41" s="42"/>
-      <c r="D41" s="42"/>
-      <c r="E41" s="42"/>
-      <c r="F41" s="42"/>
-      <c r="G41" s="42"/>
-      <c r="H41" s="42"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="28"/>
     </row>
     <row r="42" spans="1:8" ht="29" customHeight="1">
-      <c r="A42" s="56" t="s">
+      <c r="A42" s="50" t="s">
         <v>179</v>
       </c>
-      <c r="B42" s="56"/>
-      <c r="C42" s="56"/>
-      <c r="D42" s="56"/>
-      <c r="E42" s="56"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="56"/>
-      <c r="H42" s="56"/>
+      <c r="B42" s="50"/>
+      <c r="C42" s="50"/>
+      <c r="D42" s="50"/>
+      <c r="E42" s="50"/>
+      <c r="F42" s="50"/>
+      <c r="G42" s="50"/>
+      <c r="H42" s="50"/>
     </row>
     <row r="43" spans="1:8" ht="29" customHeight="1">
-      <c r="A43" s="57" t="s">
+      <c r="A43" s="51" t="s">
         <v>180</v>
       </c>
-      <c r="B43" s="57"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
+      <c r="B43" s="51"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="51"/>
+      <c r="E43" s="51"/>
+      <c r="F43" s="51"/>
+      <c r="G43" s="51"/>
+      <c r="H43" s="51"/>
     </row>
     <row r="44" spans="1:8" ht="29" customHeight="1">
-      <c r="A44" s="56" t="s">
+      <c r="A44" s="50" t="s">
         <v>181</v>
       </c>
-      <c r="B44" s="56"/>
-      <c r="C44" s="56"/>
-      <c r="D44" s="56"/>
-      <c r="E44" s="56"/>
-      <c r="F44" s="56"/>
-      <c r="G44" s="56"/>
-      <c r="H44" s="56"/>
+      <c r="B44" s="50"/>
+      <c r="C44" s="50"/>
+      <c r="D44" s="50"/>
+      <c r="E44" s="50"/>
+      <c r="F44" s="50"/>
+      <c r="G44" s="50"/>
+      <c r="H44" s="50"/>
     </row>
     <row r="45" spans="1:8" ht="29" customHeight="1">
-      <c r="A45" s="57" t="s">
+      <c r="A45" s="51" t="s">
         <v>182</v>
       </c>
-      <c r="B45" s="57"/>
-      <c r="C45" s="57"/>
-      <c r="D45" s="57"/>
-      <c r="E45" s="57"/>
-      <c r="F45" s="57"/>
-      <c r="G45" s="57"/>
-      <c r="H45" s="57"/>
+      <c r="B45" s="51"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="51"/>
+      <c r="E45" s="51"/>
+      <c r="F45" s="51"/>
+      <c r="G45" s="51"/>
+      <c r="H45" s="51"/>
     </row>
     <row r="46" spans="1:8" ht="29" customHeight="1">
-      <c r="A46" s="56" t="s">
+      <c r="A46" s="50" t="s">
         <v>183</v>
       </c>
-      <c r="B46" s="56"/>
-      <c r="C46" s="56"/>
-      <c r="D46" s="56"/>
-      <c r="E46" s="56"/>
-      <c r="F46" s="56"/>
-      <c r="G46" s="56"/>
-      <c r="H46" s="56"/>
+      <c r="B46" s="50"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="50"/>
+      <c r="E46" s="50"/>
+      <c r="F46" s="50"/>
+      <c r="G46" s="50"/>
+      <c r="H46" s="50"/>
     </row>
     <row r="47" spans="1:8" ht="14.5">
       <c r="A47" s="11"/>
@@ -17084,50 +17106,50 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="A42:H42"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="C6:H7"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:H9"/>
+    <mergeCell ref="A10:B11"/>
+    <mergeCell ref="C10:H11"/>
+    <mergeCell ref="A12:B13"/>
+    <mergeCell ref="C12:H13"/>
+    <mergeCell ref="A14:B15"/>
+    <mergeCell ref="C14:H15"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:H34"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="C35:H35"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="C36:H36"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="C37:H37"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="A33:H33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="A14:B15"/>
-    <mergeCell ref="C14:H15"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:H9"/>
-    <mergeCell ref="A10:B11"/>
-    <mergeCell ref="C10:H11"/>
-    <mergeCell ref="A12:B13"/>
-    <mergeCell ref="C12:H13"/>
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="C6:H7"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A46:H46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Feature/update UI authen (#137)
* review talent candidate

* fix sidebar

* fix all sidebar

* ui v2

* fe v2

* ui admin v3

* review v1

* fix bug update department

* sample account management

* update fe for account manage and depart

* ui monitoring

* Update authentication UI and documentation

* replace position file md

* remove block remove auto hm passsed

* sync with hoang

* sync potential candidate v1

* enhance ui for candidate potential screen

* update UI for potential candidate detail

* potential candidate v2 and potential candidate overal

* overall list candidate

* recommend suggest and overal v2 potential candidate

* update layout application detail

* Update docs

* ui for edit account admin

* create account and department

* audit log

* docs for audit log

* update ui adudit log

* layout for application and potential candidate application

* layout recommend and job posting

* docs bug

* review flow
</commit_message>
<xml_diff>
--- a/docs/members/linhdn/Professional_Bug_Tracker_Template.xlsx
+++ b/docs/members/linhdn/Professional_Bug_Tracker_Template.xlsx
@@ -19,7 +19,7 @@
     <sheet name="DanhMuc" sheetId="4" r:id="rId4"/>
     <sheet name="Huong dan" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -4101,19 +4101,61 @@
       <c r="X14" s="4"/>
       <c r="Y14" s="4"/>
     </row>
-    <row r="15" spans="1:25" ht="28" customHeight="1">
-      <c r="A15" s="2"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
+    <row r="15" spans="1:25" ht="110" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B08</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OTP đăng ký/quên mật khẩu: giao diện ghi "hiệu lực 15 phút" nhưng code chỉ cho 1 phút</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registration</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1 - Cao</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K15" s="2"/>
-      <c r="L15" s="5"/>
+      <c r="L15" s="5">
+        <v>46326</v>
+      </c>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
@@ -4126,27 +4168,96 @@
         <v/>
       </c>
       <c r="R15" s="6"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
-      <c r="U15" s="4"/>
-      <c r="V15" s="2"/>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Vào /register, nhập thông tin hợp lệ, bấm "Gửi mã xác minh".
+2. Đọc hướng dẫn trên /register/otp ("Mã có hiệu lực trong 15 phút").
+3. Đợi khoảng 2 phút rồi nhập đúng mã OTP trong email.
+(Tương tự với /forgot-password → /reset-password/otp)</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mã bị coi là hết hạn sau 1 phút; trang báo "Yêu cầu đăng ký đã hết hạn" và quay về /register (hoặc /forgot-password).</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thời hạn OTP trên giao diện và trong code giống nhau (theo SRS); nhập mã trong thời hạn ghi trên màn hình vẫn hợp lệ.</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RegistrationVerificationService.java:26 (OTP_LIFETIME = 1 phút); PasswordRecoveryService.java:25; auth/register-otp.html:14; auth/reset-password-otp.html:14; auth/forgot-password.html:15</t>
+        </is>
+      </c>
       <c r="W15" s="2"/>
-      <c r="X15" s="4"/>
-      <c r="Y15" s="4"/>
-    </row>
-    <row r="16" spans="1:25" ht="28" customHeight="1">
-      <c r="A16" s="2"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
+      <c r="X15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hằng số OTP_LIFETIME = Duration.ofMinutes(1) không khớp text cứng "15 phút" trong template.</t>
+        </is>
+      </c>
+      <c r="Y15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Liên quan B09, B10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="110" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B09</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nút "Gửi lại mã xác minh" ở bước đăng ký không bao giờ gửi được mã mới</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registration</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1 - Cao</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K16" s="2"/>
-      <c r="L16" s="5"/>
+      <c r="L16" s="5">
+        <v>46326</v>
+      </c>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
@@ -4159,27 +4270,95 @@
         <v/>
       </c>
       <c r="R16" s="6"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
-      <c r="V16" s="2"/>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Đăng ký tài khoản, sang /register/otp.
+2. Chờ hết đếm ngược 1 phút để nút "Gửi lại mã xác minh" bật lên.
+3. Bấm "Gửi lại mã xác minh".</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không gửi mã mới; bị chuyển về /register với lỗi "Yêu cầu đăng kí đã hết hạn. Vui lòng đăng kí lại", phải nhập lại mật khẩu.</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sau thời gian chờ, hệ thống gửi OTP mới cho email đang chờ xác minh và giữ người dùng ở bước nhập mã.</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RegistrationVerificationService.java:26-27, :80 (resendOtp), :154-155, :159 (requirePending)</t>
+        </is>
+      </c>
       <c r="W16" s="2"/>
-      <c r="X16" s="4"/>
-      <c r="Y16" s="4"/>
-    </row>
-    <row r="17" spans="1:25" ht="28" customHeight="1">
-      <c r="A17" s="2"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
+      <c r="X16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESEND_DELAY (1 phút) bằng đúng OTP_LIFETIME (1 phút) và resendOtp() gọi requirePending() trước, nên lúc nút vừa bật thì phiên đăng ký đã hết hạn.</t>
+        </is>
+      </c>
+      <c r="Y16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Luồng quên mật khẩu gửi lại qua POST /forgot-password nên không bị lỗi này.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:25" ht="110" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B10</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đặt lại mật khẩu: sau khi xác minh OTP chỉ còn phần thời gian còn lại của OTP (dưới 1 phút) để nhập mật khẩu mới</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auth / Login</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 - Trung bình</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K17" s="2"/>
-      <c r="L17" s="5"/>
+      <c r="L17" s="5">
+        <v>46326</v>
+      </c>
       <c r="M17" s="5"/>
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
@@ -4192,27 +4371,95 @@
         <v/>
       </c>
       <c r="R17" s="6"/>
-      <c r="S17" s="4"/>
-      <c r="T17" s="4"/>
-      <c r="U17" s="4"/>
-      <c r="V17" s="2"/>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Vào /forgot-password, nhập email, nhận OTP.
+2. Nhập đúng OTP ở khoảng giây thứ 40.
+3. Ở /reset-password, mất hơn 20 giây để nhập mật khẩu mới rồi bấm lưu.</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bị đẩy về /forgot-password với lỗi "Yêu cầu đặt lại mật khẩu không hợp lệ hoặc đã hết hạn", phải yêu cầu mã mới.</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sau khi OTP được xác minh, người dùng có một khoảng thời gian riêng, hợp lý để đặt mật khẩu mới.</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PasswordRecoveryService.java:158 (changePassword(..., state.expiresAt)), :187 (liveState); PasswordResetService.java:114</t>
+        </is>
+      </c>
       <c r="W17" s="2"/>
-      <c r="X17" s="4"/>
-      <c r="Y17" s="4"/>
-    </row>
-    <row r="18" spans="1:25" ht="28" customHeight="1">
-      <c r="A18" s="2"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bước đặt mật khẩu dùng chung mốc expiresAt của OTP (lúc gửi + 1 phút), không cấp thời hạn mới sau khi xác minh.</t>
+        </is>
+      </c>
+      <c r="Y17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Liên quan B08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:25" ht="110" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B11</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quên mật khẩu tiết lộ email nào đã có tài khoản và trạng thái tài khoản (account enumeration)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 - Trung bình</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K18" s="2"/>
-      <c r="L18" s="5"/>
+      <c r="L18" s="5">
+        <v>46326</v>
+      </c>
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
@@ -4225,27 +4472,95 @@
         <v/>
       </c>
       <c r="R18" s="6"/>
-      <c r="S18" s="4"/>
-      <c r="T18" s="4"/>
-      <c r="U18" s="4"/>
-      <c r="V18" s="2"/>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Mở /forgot-password.
+2. Nhập một email chưa đăng ký, bấm gửi.
+3. Nhập email của một tài khoản Inactive, bấm gửi.</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bước 2 báo "Không có tài khoản sử dụng email này"; bước 3 báo "Tài khoản này hiện không hoạt động". Người ngoài dò được email nào tồn tại.</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luôn hiện cùng một thông báo trung tính (vd: "Nếu email tồn tại, mã xác minh sẽ được gửi").</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PasswordResetService.java:66 (EMAIL_NOT_FOUND), :73 (ACCOUNT_NOT_ACTIVE); auth/fragments.html:134-135</t>
+        </is>
+      </c>
       <c r="W18" s="2"/>
-      <c r="X18" s="4"/>
-      <c r="Y18" s="4"/>
-    </row>
-    <row r="19" spans="1:25" ht="28" customHeight="1">
-      <c r="A19" s="2"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
+      <c r="X18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">findActiveAccount() ném lỗi riêng cho từng trường hợp và hiển thị thẳng lên form.</t>
+        </is>
+      </c>
+      <c r="Y18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Cần thống nhất với SRS / test case hiện có trước khi sửa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:25" ht="110" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B12</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi mật khẩu / đặt lại mật khẩu không đăng xuất các phiên đăng nhập khác</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 - Trung bình</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K19" s="2"/>
-      <c r="L19" s="5"/>
+      <c r="L19" s="5">
+        <v>46326</v>
+      </c>
       <c r="M19" s="5"/>
       <c r="N19" s="5"/>
       <c r="O19" s="5"/>
@@ -4258,27 +4573,95 @@
         <v/>
       </c>
       <c r="R19" s="6"/>
-      <c r="S19" s="4"/>
-      <c r="T19" s="4"/>
-      <c r="U19" s="4"/>
-      <c r="V19" s="2"/>
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Đăng nhập cùng một tài khoản trên trình duyệt A và trình duyệt B.
+2. Ở trình duyệt A, đổi mật khẩu tại /profile (hoặc đặt lại qua /forgot-password).
+3. Ở trình duyệt B, tiếp tục thao tác.</t>
+        </is>
+      </c>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trình duyệt B vẫn dùng được bình thường với phiên cũ.</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Các phiên khác của tài khoản bị vô hiệu hóa sau khi đổi / đặt lại mật khẩu.</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AccountSessionGuardFilter.java (chỉ kiểm tra AccountStatus và Role); UserProfileService.java:116; PasswordResetService.java:94</t>
+        </is>
+      </c>
       <c r="W19" s="2"/>
-      <c r="X19" s="4"/>
-      <c r="Y19" s="4"/>
-    </row>
-    <row r="20" spans="1:25" ht="28" customHeight="1">
-      <c r="A20" s="2"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
+      <c r="X19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Session guard không kiểm tra thay đổi mật khẩu; không có SessionRegistry để hủy các phiên cũ.</t>
+        </is>
+      </c>
+      <c r="Y19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:25" ht="110" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B13</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đăng nhập không giới hạn số lần nhập sai mật khẩu (chống brute-force)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auth / Login</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 - Trung bình</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K20" s="2"/>
-      <c r="L20" s="5"/>
+      <c r="L20" s="5">
+        <v>46326</v>
+      </c>
       <c r="M20" s="5"/>
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
@@ -4291,27 +4674,94 @@
         <v/>
       </c>
       <c r="R20" s="6"/>
-      <c r="S20" s="4"/>
-      <c r="T20" s="4"/>
-      <c r="U20" s="4"/>
-      <c r="V20" s="2"/>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Mở /login.
+2. Nhập đúng username, sai mật khẩu liên tục nhiều lần (vd 50 lần).</t>
+        </is>
+      </c>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lần nào cũng chỉ báo sai thông tin; không khóa tạm, không captcha, không giới hạn tốc độ.</t>
+        </is>
+      </c>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sau N lần sai liên tiếp (theo SRS) thì tạm khóa hoặc bắt chờ trước khi thử lại (OTP đã giới hạn 5 lần nhưng mật khẩu thì chưa).</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SecurityConfig.java:167-172 (formLogin chỉ có failureUrl); project không có handler đếm số lần đăng nhập sai</t>
+        </is>
+      </c>
       <c r="W20" s="2"/>
-      <c r="X20" s="4"/>
-      <c r="Y20" s="4"/>
-    </row>
-    <row r="21" spans="1:25" ht="28" customHeight="1">
-      <c r="A21" s="2"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
+      <c r="X20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa cài cơ chế chống brute-force cho form login.</t>
+        </is>
+      </c>
+      <c r="Y20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Cần xác nhận yêu cầu NFR trong SRS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:25" ht="110" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B14</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API thông báo /api/notifications/** bị tắt CSRF dù xác thực bằng session cookie</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 - Thấp</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K21" s="2"/>
-      <c r="L21" s="5"/>
+      <c r="L21" s="5">
+        <v>46326</v>
+      </c>
       <c r="M21" s="5"/>
       <c r="N21" s="5"/>
       <c r="O21" s="5"/>
@@ -4324,27 +4774,94 @@
         <v/>
       </c>
       <c r="R21" s="6"/>
-      <c r="S21" s="4"/>
-      <c r="T21" s="4"/>
-      <c r="U21" s="4"/>
-      <c r="V21" s="2"/>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Đăng nhập RMS.
+2. Mở một trang web khác có form tự submit POST tới http://localhost:8081/api/notifications/read-all.</t>
+        </is>
+      </c>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request được chấp nhận; toàn bộ thông báo của người dùng bị đánh dấu đã đọc mà người dùng không thao tác.</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Endpoint thay đổi dữ liệu dùng session cookie phải được bảo vệ CSRF như các form khác.</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SecurityConfig.java:65-66 (csrf.ignoringRequestMatchers("/api/**")); NotificationApiController.java:64, :75</t>
+        </is>
+      </c>
       <c r="W21" s="2"/>
-      <c r="X21" s="4"/>
-      <c r="Y21" s="4"/>
-    </row>
-    <row r="22" spans="1:25" ht="28" customHeight="1">
-      <c r="A22" s="2"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
+      <c r="X21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bỏ CSRF cho toàn bộ /api/** trong khi API vẫn dùng session của form login.</t>
+        </is>
+      </c>
+      <c r="Y21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Ảnh hưởng hiện tại thấp nhưng sẽ nguy hiểm nếu thêm API ghi dữ liệu khác dưới /api.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:25" ht="110" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B15</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đổi mật khẩu cho phép mật khẩu mới trùng mật khẩu hiện tại</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account Management</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validation</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 - Thấp</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K22" s="2"/>
-      <c r="L22" s="5"/>
+      <c r="L22" s="5">
+        <v>46326</v>
+      </c>
       <c r="M22" s="5"/>
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
@@ -4357,27 +4874,95 @@
         <v/>
       </c>
       <c r="R22" s="6"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
-      <c r="V22" s="2"/>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Đăng nhập, mở /profile → Đổi mật khẩu.
+2. Nhập mật khẩu hiện tại; mật khẩu mới và xác nhận đều giống mật khẩu hiện tại.
+3. Lưu.</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Báo "Đã đổi mật khẩu." dù mật khẩu không thay đổi.</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Báo lỗi "Mật khẩu mới phải khác mật khẩu hiện tại".</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UserProfileService.java:116-125; UserProfileController.java (changePasswordJson, changePasswordForm)</t>
+        </is>
+      </c>
       <c r="W22" s="2"/>
-      <c r="X22" s="4"/>
-      <c r="Y22" s="4"/>
-    </row>
-    <row r="23" spans="1:25" ht="28" customHeight="1">
-      <c r="A23" s="2"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
+      <c r="X22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chỉ kiểm tra mật khẩu hiện tại đúng và xác nhận khớp, không so sánh mật khẩu mới với mật khẩu cũ.</t>
+        </is>
+      </c>
+      <c r="Y22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Cần xác nhận rule trong SRS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:25" ht="110" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B16</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Người dùng đã đăng nhập vẫn mở được /login và /register, có thể tạo thêm tài khoản ứng viên</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auth / Login</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trivial</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 - Thấp</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K23" s="2"/>
-      <c r="L23" s="5"/>
+      <c r="L23" s="5">
+        <v>46326</v>
+      </c>
       <c r="M23" s="5"/>
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
@@ -4390,27 +4975,94 @@
         <v/>
       </c>
       <c r="R23" s="6"/>
-      <c r="S23" s="4"/>
-      <c r="T23" s="4"/>
-      <c r="U23" s="4"/>
-      <c r="V23" s="2"/>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Đăng nhập bằng bất kỳ tài khoản nào.
+2. Truy cập trực tiếp /login hoặc /register.</t>
+        </is>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Form đăng nhập / đăng ký vẫn hiển thị; có thể đăng ký tài khoản mới trong khi phiên cũ vẫn còn.</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Người dùng đã đăng nhập được chuyển hướng về /dashboard.</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AuthController.java:9-12; RegistrationController.java:26-32; SecurityConfig.java:84-86 (permitAll)</t>
+        </is>
+      </c>
       <c r="W23" s="2"/>
-      <c r="X23" s="4"/>
-      <c r="Y23" s="4"/>
-    </row>
-    <row r="24" spans="1:25" ht="28" customHeight="1">
-      <c r="A24" s="2"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
+      <c r="X23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controller không kiểm tra trạng thái đã đăng nhập trước khi trả về form.</t>
+        </is>
+      </c>
+      <c r="Y23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:25" ht="110" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B17</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">System Admin có thể tự vô hiệu hóa hoặc tự đổi role của chính mình, không chặn "admin cuối cùng"</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account Management</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1 - Cao</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K24" s="2"/>
-      <c r="L24" s="5"/>
+      <c r="L24" s="5">
+        <v>46326</v>
+      </c>
       <c r="M24" s="5"/>
       <c r="N24" s="5"/>
       <c r="O24" s="5"/>
@@ -4423,27 +5075,94 @@
         <v/>
       </c>
       <c r="R24" s="6"/>
-      <c r="S24" s="4"/>
-      <c r="T24" s="4"/>
-      <c r="U24" s="4"/>
-      <c r="V24" s="2"/>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Đăng nhập bằng System Admin (admin duy nhất).
+2. Vào /admin/accounts, bấm Vô hiệu hóa ở chính tài khoản mình (hoặc Sửa → đổi role sang HR / status Inactive).</t>
+        </is>
+      </c>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thao tác thành công; request kế tiếp bị đăng xuất (session-expired) và hệ thống không còn ai có quyền quản trị.</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không cho admin tự vô hiệu hóa / tự hạ quyền, và không cho vô hiệu hóa / hạ quyền System Admin Active cuối cùng.</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AccountListService.java:172 (deactivateScoped); AccountManagementService.java:161 (update)</t>
+        </is>
+      </c>
       <c r="W24" s="2"/>
-      <c r="X24" s="4"/>
-      <c r="Y24" s="4"/>
-    </row>
-    <row r="25" spans="1:25" ht="28" customHeight="1">
-      <c r="A25" s="2"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
+      <c r="X24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không kiểm tra userId trùng người đang thao tác, cũng không đếm số System Admin Active còn lại.</t>
+        </is>
+      </c>
+      <c r="Y24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Liên quan B20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:25" ht="110" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B18</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kích hoạt lại Hiring Manager bỏ qua rule "mỗi phòng ban tối đa 1 HM Active"</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account Management</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 - Trung bình</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K25" s="2"/>
-      <c r="L25" s="5"/>
+      <c r="L25" s="5">
+        <v>46326</v>
+      </c>
       <c r="M25" s="5"/>
       <c r="N25" s="5"/>
       <c r="O25" s="5"/>
@@ -4456,27 +5175,95 @@
         <v/>
       </c>
       <c r="R25" s="6"/>
-      <c r="S25" s="4"/>
-      <c r="T25" s="4"/>
-      <c r="U25" s="4"/>
-      <c r="V25" s="2"/>
+      <c r="S25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Phòng ban X có HM A. Vô hiệu hóa A.
+2. Tạo (hoặc đổi role) tài khoản B thành Hiring Manager của phòng X.
+3. Vào /admin/accounts, bấm Kích hoạt lại A.</t>
+        </is>
+      </c>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A được kích hoạt; phòng X có 2 Hiring Manager Active.</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chặn kích hoạt và báo "Phòng ban đã có Hiring Manager. Hãy đổi trưởng phòng trước." như khi tạo / sửa tài khoản.</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AccountListService.java:154 (activateScoped); AccountManagementService.java:108 (checkSingleHiringManager không được gọi khi kích hoạt)</t>
+        </is>
+      </c>
       <c r="W25" s="2"/>
-      <c r="X25" s="4"/>
-      <c r="Y25" s="4"/>
-    </row>
-    <row r="26" spans="1:25" ht="28" customHeight="1">
-      <c r="A26" s="2"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+      <c r="X25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nút kích hoạt đi qua AccountListService, không gọi checkSingleHiringManager.</t>
+        </is>
+      </c>
+      <c r="Y25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Liên quan B19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:25" ht="110" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B19</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vô hiệu hóa Hiring Manager không gỡ vai trò trưởng phòng (Department.Manager vẫn trỏ tới tài khoản Inactive)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account Management</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Database</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 - Trung bình</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K26" s="2"/>
-      <c r="L26" s="5"/>
+      <c r="L26" s="5">
+        <v>46326</v>
+      </c>
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
       <c r="O26" s="5"/>
@@ -4489,27 +5276,95 @@
         <v/>
       </c>
       <c r="R26" s="6"/>
-      <c r="S26" s="4"/>
-      <c r="T26" s="4"/>
-      <c r="U26" s="4"/>
-      <c r="V26" s="2"/>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Phòng ban X có trưởng phòng là HM A.
+2. Vô hiệu hóa A (nút toggle, hoặc Sửa → status Inactive, giữ nguyên role).
+3. Tạo HM mới B cho phòng X rồi xem trang phòng ban X.</t>
+        </is>
+      </c>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phòng X vẫn hiển thị trưởng phòng là A (Inactive); B không được tự gán làm trưởng phòng.</t>
+        </is>
+      </c>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khi trưởng phòng bị vô hiệu hóa thì gỡ Department.Manager (hoặc chặn cho tới khi đổi trưởng phòng); HM mới được gán làm trưởng phòng.</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AccountListService.java:172 (deactivateScoped); AccountManagementService.java:185 (chỉ gỡ manager khi đổi role / phòng ban); create() chỉ gán manager khi đang null</t>
+        </is>
+      </c>
       <c r="W26" s="2"/>
-      <c r="X26" s="4"/>
-      <c r="Y26" s="4"/>
-    </row>
-    <row r="27" spans="1:25" ht="28" customHeight="1">
-      <c r="A27" s="2"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
+      <c r="X26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ManagerId chỉ được xử lý khi role hoặc phòng ban thay đổi, bỏ qua trường hợp chuyển sang Inactive.</t>
+        </is>
+      </c>
+      <c r="Y26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Liên quan B18.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:25" ht="110" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B20</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Sửa phòng ban" cho chọn cả System Admin / Director / HR làm trưởng phòng và tự đổi họ thành Hiring Manager</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account Management</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1 - Cao</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K27" s="2"/>
-      <c r="L27" s="5"/>
+      <c r="L27" s="5">
+        <v>46326</v>
+      </c>
       <c r="M27" s="5"/>
       <c r="N27" s="5"/>
       <c r="O27" s="5"/>
@@ -4522,27 +5377,95 @@
         <v/>
       </c>
       <c r="R27" s="6"/>
-      <c r="S27" s="4"/>
-      <c r="T27" s="4"/>
-      <c r="U27" s="4"/>
-      <c r="V27" s="2"/>
+      <c r="S27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Đăng nhập System Admin (tài khoản admin thuộc phòng ban X).
+2. Vào /admin/departments → Sửa phòng ban X.
+3. Ở ô Trưởng phòng chọn chính tài khoản admin (hoặc một Director / HR) → Lưu.</t>
+        </is>
+      </c>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Người được chọn bị đổi role thành Hiring Manager (admin mất quyền quản trị, Director mất quyền duyệt); trưởng phòng cũ bị đổi thành Interviewer.</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Danh sách chọn chỉ gồm tài khoản phù hợp (vd Interviewer / Hiring Manager) hoặc có xác nhận trước khi đổi role; không bao giờ tự đổi role System Admin / Director.</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DepartmentService.java:57-61 (managerChoices lọc theo INTERNAL_ROLE_NAMES), :96-104 (đổi role trưởng phòng mới và cũ)</t>
+        </is>
+      </c>
       <c r="W27" s="2"/>
-      <c r="X27" s="4"/>
-      <c r="Y27" s="4"/>
-    </row>
-    <row r="28" spans="1:25" ht="28" customHeight="1">
-      <c r="A28" s="2"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">managerChoices lấy mọi role nội bộ đang Active trong phòng ban; update() gán role Hiring Manager cho bất kỳ ai được chọn.</t>
+        </is>
+      </c>
+      <c r="Y27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Liên quan B17.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:25" ht="110" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B21</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validation họ tên / SĐT không thống nhất giữa Admin tạo tài khoản, Đăng ký và Cập nhật hồ sơ</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account Management</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validation</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 - Thấp</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K28" s="2"/>
-      <c r="L28" s="5"/>
+      <c r="L28" s="5">
+        <v>46326</v>
+      </c>
       <c r="M28" s="5"/>
       <c r="N28" s="5"/>
       <c r="O28" s="5"/>
@@ -4555,27 +5478,94 @@
         <v/>
       </c>
       <c r="R28" s="6"/>
-      <c r="S28" s="4"/>
-      <c r="T28" s="4"/>
-      <c r="U28" s="4"/>
-      <c r="V28" s="2"/>
+      <c r="S28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Admin tạo tài khoản với họ tên "A" (1 ký tự) hoặc "Nguyễn 123", SĐT 18 ký tự có chữ (hoặc ứng viên tự đăng ký với họ tên "A1").
+2. Đăng nhập bằng tài khoản đó, vào /profile, bấm Lưu thông tin.</t>
+        </is>
+      </c>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tạo / đăng ký thành công, nhưng khi tự cập nhật hồ sơ thì bị báo họ tên / SĐT không hợp lệ.</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cùng một rule cho họ tên (2–100 ký tự, chỉ chữ cái...) và SĐT (≤15 ký tự, chỉ số và + - ( ) khoảng trắng) ở mọi màn hình.</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CreateAccountRequest.java:9-23; UpdateAccountRequest.java:24; RegisterAccountRequest.java:14-16; UpdateProfileRequest.java:15-23</t>
+        </is>
+      </c>
       <c r="W28" s="2"/>
-      <c r="X28" s="4"/>
-      <c r="Y28" s="4"/>
-    </row>
-    <row r="29" spans="1:25" ht="28" customHeight="1">
-      <c r="A29" s="2"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
+      <c r="X28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mỗi DTO tự khai báo ràng buộc riêng; chỉ UpdateProfileRequest có @Pattern và giới hạn SĐT 15 ký tự.</t>
+        </is>
+      </c>
+      <c r="Y28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:25" ht="110" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B22</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tên đăng nhập không có ràng buộc định dạng (cho phép khoảng trắng, dấu tiếng Việt, ký tự đặc biệt)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registration</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validation</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 - Thấp</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K29" s="2"/>
-      <c r="L29" s="5"/>
+      <c r="L29" s="5">
+        <v>46326</v>
+      </c>
       <c r="M29" s="5"/>
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
@@ -4588,27 +5578,95 @@
         <v/>
       </c>
       <c r="R29" s="6"/>
-      <c r="S29" s="4"/>
-      <c r="T29" s="4"/>
-      <c r="U29" s="4"/>
-      <c r="V29" s="2"/>
+      <c r="S29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Mở /register (hoặc Admin → Tạo tài khoản).
+2. Nhập tên đăng nhập "nguyễn văn a" hoặc "&lt;b&gt;abc&lt;/b&gt;", các trường khác hợp lệ.
+3. Gửi.</t>
+        </is>
+      </c>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Được chấp nhận; username chứa khoảng trắng / ký tự đặc biệt.</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Username chỉ gồm chữ không dấu, số và một số ký tự cho phép (vd . _ -), có độ dài tối thiểu, theo SRS.</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RegisterAccountRequest.java:18-20; CreateAccountRequest.java:13-15</t>
+        </is>
+      </c>
       <c r="W29" s="2"/>
-      <c r="X29" s="4"/>
-      <c r="Y29" s="4"/>
-    </row>
-    <row r="30" spans="1:25" ht="28" customHeight="1">
-      <c r="A30" s="2"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
+      <c r="X29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chỉ có @NotBlank và @Size(max = 50), không có @Pattern.</t>
+        </is>
+      </c>
+      <c r="Y29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Cần thống nhất format trong SRS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="1:25" ht="110" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B23</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vô hiệu hóa phòng ban không kiểm tra tài khoản, requisition và tin tuyển dụng đang hoạt động</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account Management</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3 - Thấp</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature/update-ui-authen</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linh (code review)</t>
+        </is>
+      </c>
       <c r="K30" s="2"/>
-      <c r="L30" s="5"/>
+      <c r="L30" s="5">
+        <v>46326</v>
+      </c>
       <c r="M30" s="5"/>
       <c r="N30" s="5"/>
       <c r="O30" s="5"/>
@@ -4621,13 +5679,38 @@
         <v/>
       </c>
       <c r="R30" s="6"/>
-      <c r="S30" s="4"/>
-      <c r="T30" s="4"/>
-      <c r="U30" s="4"/>
-      <c r="V30" s="2"/>
+      <c r="S30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Phòng ban X có tài khoản Active, requisition đang chờ duyệt và tin đang Published.
+2. Vào /admin/departments, bấm Vô hiệu hóa phòng X.</t>
+        </is>
+      </c>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vô hiệu hóa ngay, không cảnh báo; nhân viên phòng X vẫn làm việc bình thường, tin vẫn nhận hồ sơ.</t>
+        </is>
+      </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cảnh báo / chặn khi phòng ban còn dữ liệu đang hoạt động, hoặc SRS mô tả rõ hệ quả.</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DepartmentService.java:124-135 (deactivate / activate / setStatus)</t>
+        </is>
+      </c>
       <c r="W30" s="2"/>
-      <c r="X30" s="4"/>
-      <c r="Y30" s="4"/>
+      <c r="X30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">setStatus() chỉ đổi DepartmentStatus, không kiểm tra dữ liệu phụ thuộc.</t>
+        </is>
+      </c>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chưa fix. Cần xác nhận nghiệp vụ.</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:25" ht="28" customHeight="1">
       <c r="A31" s="2"/>

</xml_diff>